<commit_message>
Fix presentation PDF and WBS font rendering
</commit_message>
<xml_diff>
--- a/Energy_Budget_WBS_Gantt.xlsx
+++ b/Energy_Budget_WBS_Gantt.xlsx
@@ -113,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -238,11 +238,99 @@
         <color rgb="00D9DEE7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00FF3B3B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FF3B3B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00FF3B3B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C7CDD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FF3B3B"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C7CDD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C7CDD6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C7CDD6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C7CDD6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C7CDD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9DEE7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C7CDD6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C7CDD6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -326,6 +414,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -749,10 +841,11 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>?? Energy Budget WBS &amp; Gantt Chart</t>
-        </is>
-      </c>
-    </row>
+          <t>Energy Budget WBS &amp; Gantt Chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -796,70 +889,70 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>10?</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4" t="n"/>
-      <c r="O3" s="4" t="n"/>
+          <t>10-&gt;</t>
+        </is>
+      </c>
+      <c r="J3" s="31" t="n"/>
+      <c r="K3" s="31" t="n"/>
+      <c r="L3" s="31" t="n"/>
+      <c r="M3" s="31" t="n"/>
+      <c r="N3" s="31" t="n"/>
+      <c r="O3" s="32" t="n"/>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>11?</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
+          <t>11-&gt;</t>
+        </is>
+      </c>
+      <c r="Q3" s="31" t="n"/>
+      <c r="R3" s="31" t="n"/>
+      <c r="S3" s="31" t="n"/>
+      <c r="T3" s="31" t="n"/>
+      <c r="U3" s="31" t="n"/>
+      <c r="V3" s="32" t="n"/>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>12?</t>
-        </is>
-      </c>
-      <c r="X3" s="6" t="n"/>
-      <c r="Y3" s="6" t="n"/>
-      <c r="Z3" s="6" t="n"/>
-      <c r="AA3" s="6" t="n"/>
-      <c r="AB3" s="6" t="n"/>
-      <c r="AC3" s="6" t="n"/>
+          <t>12-&gt;</t>
+        </is>
+      </c>
+      <c r="X3" s="33" t="n"/>
+      <c r="Y3" s="33" t="n"/>
+      <c r="Z3" s="33" t="n"/>
+      <c r="AA3" s="33" t="n"/>
+      <c r="AB3" s="33" t="n"/>
+      <c r="AC3" s="34" t="n"/>
       <c r="AD3" s="3" t="inlineStr">
         <is>
-          <t>13?</t>
-        </is>
-      </c>
-      <c r="AE3" s="4" t="n"/>
-      <c r="AF3" s="4" t="n"/>
-      <c r="AG3" s="4" t="n"/>
-      <c r="AH3" s="4" t="n"/>
-      <c r="AI3" s="4" t="n"/>
-      <c r="AJ3" s="4" t="n"/>
+          <t>13-&gt;</t>
+        </is>
+      </c>
+      <c r="AE3" s="31" t="n"/>
+      <c r="AF3" s="31" t="n"/>
+      <c r="AG3" s="31" t="n"/>
+      <c r="AH3" s="31" t="n"/>
+      <c r="AI3" s="31" t="n"/>
+      <c r="AJ3" s="32" t="n"/>
       <c r="AK3" s="3" t="inlineStr">
         <is>
-          <t>14?</t>
-        </is>
-      </c>
-      <c r="AL3" s="4" t="n"/>
-      <c r="AM3" s="4" t="n"/>
-      <c r="AN3" s="4" t="n"/>
-      <c r="AO3" s="4" t="n"/>
-      <c r="AP3" s="4" t="n"/>
-      <c r="AQ3" s="4" t="n"/>
+          <t>14-&gt;</t>
+        </is>
+      </c>
+      <c r="AL3" s="31" t="n"/>
+      <c r="AM3" s="31" t="n"/>
+      <c r="AN3" s="31" t="n"/>
+      <c r="AO3" s="31" t="n"/>
+      <c r="AP3" s="31" t="n"/>
+      <c r="AQ3" s="32" t="n"/>
       <c r="AR3" s="3" t="inlineStr">
         <is>
-          <t>15?</t>
-        </is>
-      </c>
-      <c r="AS3" s="4" t="n"/>
-      <c r="AT3" s="4" t="n"/>
-      <c r="AU3" s="4" t="n"/>
-      <c r="AV3" s="4" t="n"/>
-      <c r="AW3" s="4" t="n"/>
-      <c r="AX3" s="4" t="n"/>
+          <t>15-&gt;</t>
+        </is>
+      </c>
+      <c r="AS3" s="31" t="n"/>
+      <c r="AT3" s="31" t="n"/>
+      <c r="AU3" s="31" t="n"/>
+      <c r="AV3" s="31" t="n"/>
+      <c r="AW3" s="31" t="n"/>
+      <c r="AX3" s="32" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="7" t="n"/>
@@ -1089,7 +1182,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1161,16 +1254,8 @@
           <t>1.1</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>?? ??</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B6" s="16" t="inlineStr"/>
+      <c r="C6" s="15" t="inlineStr"/>
       <c r="D6" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1241,16 +1326,8 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>???? ??</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B7" s="16" t="inlineStr"/>
+      <c r="C7" s="15" t="inlineStr"/>
       <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1327,14 +1404,10 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>WBS ??</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">WBS </t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr"/>
       <c r="D8" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1411,14 +1484,10 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>??/??/BONUS ??</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">//BONUS </t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr"/>
       <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1489,16 +1558,8 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B10" s="21" t="inlineStr"/>
+      <c r="C10" s="20" t="inlineStr"/>
       <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -1524,7 +1585,7 @@
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="P10" s="13" t="n"/>
@@ -1571,7 +1632,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1645,14 +1706,10 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr"/>
       <c r="D12" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1725,14 +1782,10 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>??? ??</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr"/>
       <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1803,16 +1856,8 @@
           <t>2.3</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>??????</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B14" s="16" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr"/>
       <c r="D14" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1883,16 +1928,8 @@
           <t>3.1</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>??? ??? ??</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B15" s="16" t="inlineStr"/>
+      <c r="C15" s="15" t="inlineStr"/>
       <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -1965,14 +2002,10 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>? ? ??? ??</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt; -&gt; -&gt;</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -2045,14 +2078,10 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>?? ?? ??? ??</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr"/>
       <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -2125,14 +2154,10 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>?? ??? ??</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr"/>
       <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Completed</t>
@@ -2205,14 +2230,10 @@
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>??/?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C19" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr"/>
       <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -2245,7 +2266,7 @@
       <c r="U19" s="13" t="n"/>
       <c r="V19" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="W19" s="14" t="n"/>
@@ -2285,7 +2306,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>?? ?? 1 ??</t>
+          <t xml:space="preserve">1 </t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -2359,14 +2380,10 @@
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr"/>
       <c r="D21" s="25" t="inlineStr">
         <is>
           <t>In progress</t>
@@ -2443,14 +2460,10 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>? ? ?? ??</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">-&gt; -&gt; </t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr"/>
       <c r="D22" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2527,14 +2540,10 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr"/>
       <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2607,14 +2616,10 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>?? ??? ??</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr"/>
       <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2685,16 +2690,8 @@
           <t>5.1</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
-        <is>
-          <t>??? ?? ???</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B25" s="16" t="inlineStr"/>
+      <c r="C25" s="15" t="inlineStr"/>
       <c r="D25" s="25" t="inlineStr">
         <is>
           <t>In progress</t>
@@ -2767,14 +2764,10 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>? ? ??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt; -&gt; -&gt;</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr"/>
       <c r="D26" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2847,14 +2840,10 @@
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>MVP ?? ?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C27" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">MVP </t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr"/>
       <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -2894,7 +2883,7 @@
       <c r="AB27" s="13" t="n"/>
       <c r="AC27" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="AD27" s="13" t="n"/>
@@ -2927,7 +2916,7 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>?? ?? 2 ??? ???</t>
+          <t xml:space="preserve">2 </t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3001,14 +2990,10 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr"/>
       <c r="D29" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3081,14 +3066,10 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr"/>
       <c r="D30" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3159,16 +3140,8 @@
           <t>6.1</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>?? ???? ??</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B31" s="16" t="inlineStr"/>
+      <c r="C31" s="15" t="inlineStr"/>
       <c r="D31" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3241,14 +3214,10 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>?? ? ? ?? ??</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">-&gt; -&gt; </t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr"/>
       <c r="D32" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3333,14 +3302,10 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr"/>
       <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3411,16 +3376,8 @@
           <t>6.4</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
-        <is>
-          <t>?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B34" s="16" t="inlineStr"/>
+      <c r="C34" s="15" t="inlineStr"/>
       <c r="D34" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3503,16 +3460,8 @@
           <t>7.1</t>
         </is>
       </c>
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>?? ?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B35" s="16" t="inlineStr"/>
+      <c r="C35" s="15" t="inlineStr"/>
       <c r="D35" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3583,16 +3532,8 @@
           <t>7.2</t>
         </is>
       </c>
-      <c r="B36" s="16" t="inlineStr">
-        <is>
-          <t>?? ?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B36" s="16" t="inlineStr"/>
+      <c r="C36" s="15" t="inlineStr"/>
       <c r="D36" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3663,16 +3604,8 @@
           <t>7.3</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
-        <is>
-          <t>?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B37" s="16" t="inlineStr"/>
+      <c r="C37" s="15" t="inlineStr"/>
       <c r="D37" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3745,14 +3678,10 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>??/?? ?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C38" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="inlineStr"/>
       <c r="D38" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -3799,7 +3728,7 @@
       <c r="AI38" s="13" t="n"/>
       <c r="AJ38" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="AK38" s="13" t="n"/>
@@ -3823,11 +3752,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>???? ?? ??</t>
-        </is>
-      </c>
+      <c r="B39" s="10" t="inlineStr"/>
       <c r="C39" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -3897,16 +3822,8 @@
           <t>8.1</t>
         </is>
       </c>
-      <c r="B40" s="16" t="inlineStr">
-        <is>
-          <t>?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B40" s="16" t="inlineStr"/>
+      <c r="C40" s="15" t="inlineStr"/>
       <c r="D40" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3983,14 +3900,10 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr"/>
       <c r="D41" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4067,14 +3980,10 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>?? ??? ?? ??</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr"/>
       <c r="D42" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4147,14 +4056,10 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>?? ??? ??</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr"/>
       <c r="D43" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4239,14 +4144,10 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>?? ?? ??? ??</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr"/>
       <c r="D44" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4317,16 +4218,8 @@
           <t>9.2</t>
         </is>
       </c>
-      <c r="B45" s="16" t="inlineStr">
-        <is>
-          <t>??? ???? ???</t>
-        </is>
-      </c>
-      <c r="C45" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B45" s="16" t="inlineStr"/>
+      <c r="C45" s="15" t="inlineStr"/>
       <c r="D45" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4399,14 +4292,10 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>README ??</t>
-        </is>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">README </t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr"/>
       <c r="D46" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4479,14 +4368,10 @@
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>???/?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C47" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t>-&gt;/</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr"/>
       <c r="D47" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -4540,7 +4425,7 @@
       <c r="AP47" s="13" t="n"/>
       <c r="AQ47" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
       <c r="AR47" s="13" t="n"/>
@@ -4557,11 +4442,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>?? ??</t>
-        </is>
-      </c>
+      <c r="B48" s="10" t="inlineStr"/>
       <c r="C48" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -4633,14 +4514,10 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>?? ?? ?? ? ?? ?? ??</t>
-        </is>
-      </c>
-      <c r="C49" s="15" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+          <t xml:space="preserve">-&gt; </t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr"/>
       <c r="D49" s="28" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4735,16 +4612,8 @@
           <t>M6</t>
         </is>
       </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>?? ??</t>
-        </is>
-      </c>
-      <c r="C50" s="20" t="inlineStr">
-        <is>
-          <t>??</t>
-        </is>
-      </c>
+      <c r="B50" s="21" t="inlineStr"/>
+      <c r="C50" s="20" t="inlineStr"/>
       <c r="D50" s="20" t="inlineStr">
         <is>
           <t>Milestone</t>
@@ -4805,7 +4674,7 @@
       <c r="AW50" s="13" t="n"/>
       <c r="AX50" s="23" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>-&gt;</t>
         </is>
       </c>
     </row>
@@ -4847,49 +4716,50 @@
     <row r="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>Energy Budget WBS &amp; Gantt Chart ???</t>
-        </is>
-      </c>
-    </row>
+          <t>Energy Budget WBS &amp; Gantt Chart -&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
         <is>
-          <t>1. WBS/Task/Status/Start Date/Finish Date? ?? ??? ?????.</t>
+          <t>1. WBS/Task/Status/Start Date/Finish Date-&gt; .</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>2. ??? ?? ??? ?? ?? ??? ?? ?????.</t>
+          <t>2. .</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="30" t="inlineStr">
         <is>
-          <t>3. ?? ??? ?? ???? ?? ?? ?????.</t>
+          <t>3. .</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="30" t="inlineStr">
         <is>
-          <t>4. ? ??? ???????.</t>
+          <t>4. -&gt; .</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="30" t="inlineStr">
         <is>
-          <t>5. ?? ???? ?? ?? 2026-05-26? ?????.</t>
+          <t>5. 2026-05-26-&gt; -&gt;.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
         <is>
-          <t>6. ??? 10?? 2026-05-12 ?? ???? 15???? ??????.</t>
+          <t>6. -&gt;102026-05-12 15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WBS owner and project timeline
</commit_message>
<xml_diff>
--- a/Energy_Budget_WBS_Gantt.xlsx
+++ b/Energy_Budget_WBS_Gantt.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS Gantt" sheetId="1" r:id="Rf2f04876c3ae44a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R7713153bd6df4963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS Gantt" sheetId="1" r:id="R085271602f764c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rbf8e628ebabd4a70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -79,6 +79,16 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE0F2FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D4ED8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FF22C55E"/>
       </x:patternFill>
     </x:fill>
@@ -89,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -100,9 +110,12 @@
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -314,7 +327,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Energy Budget WBS and Gantt Chart</x:v>
+        <x:v>Energy Budget WBS &amp; Gantt Chart</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str"/>
       <x:c r="C1" s="2" t="str"/>
@@ -473,7 +486,7 @@
         <x:v>W</x:v>
       </x:c>
       <x:c r="H3" s="4" t="str">
-        <x:v>Progress</x:v>
+        <x:v>%</x:v>
       </x:c>
       <x:c r="I3" s="4" t="str">
         <x:v>1</x:v>
@@ -607,7 +620,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>기획과 문제 정의</x:v>
+        <x:v>기획 및 문제 정의</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
         <x:v>-</x:v>
@@ -675,10 +688,10 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>프로젝트 비전 정리</x:v>
+        <x:v>프로젝트 주제 확정</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D5" s="8" t="str">
         <x:v>Completed</x:v>
@@ -687,17 +700,17 @@
         <x:v>2026-05-12</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-12</x:v>
       </x:c>
       <x:c r="G5" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H5" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="I5" t="str"/>
       <x:c r="J5" s="9" t="str"/>
-      <x:c r="K5" s="9" t="str"/>
+      <x:c r="K5" t="str"/>
       <x:c r="L5" t="str"/>
       <x:c r="M5" t="str"/>
       <x:c r="N5" t="str"/>
@@ -743,19 +756,19 @@
         <x:v>1.2</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>사용자 시나리오 정리</x:v>
+        <x:v>비전과 문제 정의 작성</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E6" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
         <x:v>2026-05-13</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:v>2026-05-14</x:v>
       </x:c>
       <x:c r="G6" t="n">
         <x:v>2</x:v>
@@ -764,9 +777,9 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="I6" t="str"/>
-      <x:c r="J6" t="str"/>
+      <x:c r="J6" s="9" t="str"/>
       <x:c r="K6" s="9" t="str"/>
-      <x:c r="L6" s="9" t="str"/>
+      <x:c r="L6" t="str"/>
       <x:c r="M6" t="str"/>
       <x:c r="N6" t="str"/>
       <x:c r="O6" t="str"/>
@@ -811,19 +824,19 @@
         <x:v>1.3</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>MoSCoW 기능 분류</x:v>
+        <x:v>사용자 시나리오 3개 작성</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D7" s="8" t="str">
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E7" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
         <x:v>2026-05-14</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G7" t="n">
         <x:v>2</x:v>
@@ -833,9 +846,9 @@
       </x:c>
       <x:c r="I7" t="str"/>
       <x:c r="J7" t="str"/>
-      <x:c r="K7" t="str"/>
+      <x:c r="K7" s="9" t="str"/>
       <x:c r="L7" s="9" t="str"/>
-      <x:c r="M7" s="9" t="str"/>
+      <x:c r="M7" t="str"/>
       <x:c r="N7" t="str"/>
       <x:c r="O7" t="str"/>
       <x:c r="P7" t="str"/>
@@ -879,22 +892,22 @@
         <x:v>1.4</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>WBS와 일정 문서 정리</x:v>
+        <x:v>MoSCoW 기능 분류</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>2026-05-16</x:v>
+        <x:v>2026-05-14</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>2026-05-18</x:v>
+        <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="G8" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H8" t="n">
         <x:v>100</x:v>
@@ -902,11 +915,11 @@
       <x:c r="I8" t="str"/>
       <x:c r="J8" t="str"/>
       <x:c r="K8" t="str"/>
-      <x:c r="L8" t="str"/>
-      <x:c r="M8" t="str"/>
-      <x:c r="N8" s="9" t="str"/>
-      <x:c r="O8" s="9" t="str"/>
-      <x:c r="P8" s="9" t="str"/>
+      <x:c r="L8" s="9" t="str"/>
+      <x:c r="M8" s="9" t="str"/>
+      <x:c r="N8" t="str"/>
+      <x:c r="O8" t="str"/>
+      <x:c r="P8" t="str"/>
       <x:c r="Q8" t="str"/>
       <x:c r="R8" t="str"/>
       <x:c r="S8" t="str"/>
@@ -943,230 +956,230 @@
       <x:c r="AX8" t="str"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6" t="str">
+      <x:c r="A9" t="str">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>WBS와 6주 일정 정리</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>2026-05-16</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>2026-05-18</x:v>
+      </x:c>
+      <x:c r="G9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I9" t="str"/>
+      <x:c r="J9" t="str"/>
+      <x:c r="K9" t="str"/>
+      <x:c r="L9" t="str"/>
+      <x:c r="M9" t="str"/>
+      <x:c r="N9" s="9" t="str"/>
+      <x:c r="O9" s="9" t="str"/>
+      <x:c r="P9" s="9" t="str"/>
+      <x:c r="Q9" t="str"/>
+      <x:c r="R9" t="str"/>
+      <x:c r="S9" t="str"/>
+      <x:c r="T9" t="str"/>
+      <x:c r="U9" t="str"/>
+      <x:c r="V9" t="str"/>
+      <x:c r="W9" t="str"/>
+      <x:c r="X9" t="str"/>
+      <x:c r="Y9" t="str"/>
+      <x:c r="Z9" t="str"/>
+      <x:c r="AA9" t="str"/>
+      <x:c r="AB9" t="str"/>
+      <x:c r="AC9" t="str"/>
+      <x:c r="AD9" t="str"/>
+      <x:c r="AE9" t="str"/>
+      <x:c r="AF9" t="str"/>
+      <x:c r="AG9" t="str"/>
+      <x:c r="AH9" t="str"/>
+      <x:c r="AI9" t="str"/>
+      <x:c r="AJ9" t="str"/>
+      <x:c r="AK9" t="str"/>
+      <x:c r="AL9" t="str"/>
+      <x:c r="AM9" t="str"/>
+      <x:c r="AN9" t="str"/>
+      <x:c r="AO9" t="str"/>
+      <x:c r="AP9" t="str"/>
+      <x:c r="AQ9" t="str"/>
+      <x:c r="AR9" t="str"/>
+      <x:c r="AS9" t="str"/>
+      <x:c r="AT9" t="str"/>
+      <x:c r="AU9" t="str"/>
+      <x:c r="AV9" t="str"/>
+      <x:c r="AW9" t="str"/>
+      <x:c r="AX9" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="str">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>1차 산출물 점검</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Milestone</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>2026-05-18</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>2026-05-18</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="str"/>
+      <x:c r="J10" s="11" t="str"/>
+      <x:c r="K10" s="11" t="str"/>
+      <x:c r="L10" s="11" t="str"/>
+      <x:c r="M10" s="11" t="str"/>
+      <x:c r="N10" s="11" t="str"/>
+      <x:c r="O10" s="11" t="str"/>
+      <x:c r="P10" s="12" t="str"/>
+      <x:c r="Q10" s="11" t="str"/>
+      <x:c r="R10" s="11" t="str"/>
+      <x:c r="S10" s="11" t="str"/>
+      <x:c r="T10" s="11" t="str"/>
+      <x:c r="U10" s="11" t="str"/>
+      <x:c r="V10" s="11" t="str"/>
+      <x:c r="W10" s="11" t="str"/>
+      <x:c r="X10" s="11" t="str"/>
+      <x:c r="Y10" s="11" t="str"/>
+      <x:c r="Z10" s="11" t="str"/>
+      <x:c r="AA10" s="11" t="str"/>
+      <x:c r="AB10" s="11" t="str"/>
+      <x:c r="AC10" s="11" t="str"/>
+      <x:c r="AD10" s="11" t="str"/>
+      <x:c r="AE10" s="11" t="str"/>
+      <x:c r="AF10" s="11" t="str"/>
+      <x:c r="AG10" s="11" t="str"/>
+      <x:c r="AH10" s="11" t="str"/>
+      <x:c r="AI10" s="11" t="str"/>
+      <x:c r="AJ10" s="11" t="str"/>
+      <x:c r="AK10" s="11" t="str"/>
+      <x:c r="AL10" s="11" t="str"/>
+      <x:c r="AM10" s="11" t="str"/>
+      <x:c r="AN10" s="11" t="str"/>
+      <x:c r="AO10" s="11" t="str"/>
+      <x:c r="AP10" s="11" t="str"/>
+      <x:c r="AQ10" s="11" t="str"/>
+      <x:c r="AR10" s="11" t="str"/>
+      <x:c r="AS10" s="11" t="str"/>
+      <x:c r="AT10" s="11" t="str"/>
+      <x:c r="AU10" s="11" t="str"/>
+      <x:c r="AV10" s="11" t="str"/>
+      <x:c r="AW10" s="11" t="str"/>
+      <x:c r="AX10" s="11" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="6" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>설계와 개발 환경</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="str">
+      <x:c r="B11" s="6" t="str">
+        <x:v>설계 및 개발 환경</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="D9" s="6" t="str">
+      <x:c r="D11" s="6" t="str">
         <x:v>Completed</x:v>
       </x:c>
-      <x:c r="E9" s="6" t="str">
+      <x:c r="E11" s="6" t="str">
         <x:v>2026-05-19</x:v>
       </x:c>
-      <x:c r="F9" s="6" t="str">
+      <x:c r="F11" s="6" t="str">
         <x:v>2026-05-25</x:v>
       </x:c>
-      <x:c r="G9" s="6" t="n">
+      <x:c r="G11" s="6" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="H9" s="6" t="n">
+      <x:c r="H11" s="6" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="I9" s="6" t="str"/>
-      <x:c r="J9" s="6" t="str"/>
-      <x:c r="K9" s="6" t="str"/>
-      <x:c r="L9" s="6" t="str"/>
-      <x:c r="M9" s="6" t="str"/>
-      <x:c r="N9" s="6" t="str"/>
-      <x:c r="O9" s="6" t="str"/>
-      <x:c r="P9" s="6" t="str"/>
-      <x:c r="Q9" s="7" t="str"/>
-      <x:c r="R9" s="7" t="str"/>
-      <x:c r="S9" s="7" t="str"/>
-      <x:c r="T9" s="7" t="str"/>
-      <x:c r="U9" s="7" t="str"/>
-      <x:c r="V9" s="7" t="str"/>
-      <x:c r="W9" s="7" t="str"/>
-      <x:c r="X9" s="6" t="str"/>
-      <x:c r="Y9" s="6" t="str"/>
-      <x:c r="Z9" s="6" t="str"/>
-      <x:c r="AA9" s="6" t="str"/>
-      <x:c r="AB9" s="6" t="str"/>
-      <x:c r="AC9" s="6" t="str"/>
-      <x:c r="AD9" s="6" t="str"/>
-      <x:c r="AE9" s="6" t="str"/>
-      <x:c r="AF9" s="6" t="str"/>
-      <x:c r="AG9" s="6" t="str"/>
-      <x:c r="AH9" s="6" t="str"/>
-      <x:c r="AI9" s="6" t="str"/>
-      <x:c r="AJ9" s="6" t="str"/>
-      <x:c r="AK9" s="6" t="str"/>
-      <x:c r="AL9" s="6" t="str"/>
-      <x:c r="AM9" s="6" t="str"/>
-      <x:c r="AN9" s="6" t="str"/>
-      <x:c r="AO9" s="6" t="str"/>
-      <x:c r="AP9" s="6" t="str"/>
-      <x:c r="AQ9" s="6" t="str"/>
-      <x:c r="AR9" s="6" t="str"/>
-      <x:c r="AS9" s="6" t="str"/>
-      <x:c r="AT9" s="6" t="str"/>
-      <x:c r="AU9" s="6" t="str"/>
-      <x:c r="AV9" s="6" t="str"/>
-      <x:c r="AW9" s="6" t="str"/>
-      <x:c r="AX9" s="6" t="str"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>2.1</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>ADR 기반 기술 선택</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D10" s="8" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>2026-05-19</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>2026-05-20</x:v>
-      </x:c>
-      <x:c r="G10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H10" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="I10" t="str"/>
-      <x:c r="J10" t="str"/>
-      <x:c r="K10" t="str"/>
-      <x:c r="L10" t="str"/>
-      <x:c r="M10" t="str"/>
-      <x:c r="N10" t="str"/>
-      <x:c r="O10" t="str"/>
-      <x:c r="P10" t="str"/>
-      <x:c r="Q10" s="9" t="str"/>
-      <x:c r="R10" s="9" t="str"/>
-      <x:c r="S10" t="str"/>
-      <x:c r="T10" t="str"/>
-      <x:c r="U10" t="str"/>
-      <x:c r="V10" t="str"/>
-      <x:c r="W10" t="str"/>
-      <x:c r="X10" t="str"/>
-      <x:c r="Y10" t="str"/>
-      <x:c r="Z10" t="str"/>
-      <x:c r="AA10" t="str"/>
-      <x:c r="AB10" t="str"/>
-      <x:c r="AC10" t="str"/>
-      <x:c r="AD10" t="str"/>
-      <x:c r="AE10" t="str"/>
-      <x:c r="AF10" t="str"/>
-      <x:c r="AG10" t="str"/>
-      <x:c r="AH10" t="str"/>
-      <x:c r="AI10" t="str"/>
-      <x:c r="AJ10" t="str"/>
-      <x:c r="AK10" t="str"/>
-      <x:c r="AL10" t="str"/>
-      <x:c r="AM10" t="str"/>
-      <x:c r="AN10" t="str"/>
-      <x:c r="AO10" t="str"/>
-      <x:c r="AP10" t="str"/>
-      <x:c r="AQ10" t="str"/>
-      <x:c r="AR10" t="str"/>
-      <x:c r="AS10" t="str"/>
-      <x:c r="AT10" t="str"/>
-      <x:c r="AU10" t="str"/>
-      <x:c r="AV10" t="str"/>
-      <x:c r="AW10" t="str"/>
-      <x:c r="AX10" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>2.2</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Expo 프로젝트 초기화</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D11" s="8" t="str">
-        <x:v>Completed</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>2026-05-20</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>2026-05-21</x:v>
-      </x:c>
-      <x:c r="G11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H11" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="I11" t="str"/>
-      <x:c r="J11" t="str"/>
-      <x:c r="K11" t="str"/>
-      <x:c r="L11" t="str"/>
-      <x:c r="M11" t="str"/>
-      <x:c r="N11" t="str"/>
-      <x:c r="O11" t="str"/>
-      <x:c r="P11" t="str"/>
-      <x:c r="Q11" t="str"/>
-      <x:c r="R11" s="9" t="str"/>
-      <x:c r="S11" s="9" t="str"/>
-      <x:c r="T11" t="str"/>
-      <x:c r="U11" t="str"/>
-      <x:c r="V11" t="str"/>
-      <x:c r="W11" t="str"/>
-      <x:c r="X11" t="str"/>
-      <x:c r="Y11" t="str"/>
-      <x:c r="Z11" t="str"/>
-      <x:c r="AA11" t="str"/>
-      <x:c r="AB11" t="str"/>
-      <x:c r="AC11" t="str"/>
-      <x:c r="AD11" t="str"/>
-      <x:c r="AE11" t="str"/>
-      <x:c r="AF11" t="str"/>
-      <x:c r="AG11" t="str"/>
-      <x:c r="AH11" t="str"/>
-      <x:c r="AI11" t="str"/>
-      <x:c r="AJ11" t="str"/>
-      <x:c r="AK11" t="str"/>
-      <x:c r="AL11" t="str"/>
-      <x:c r="AM11" t="str"/>
-      <x:c r="AN11" t="str"/>
-      <x:c r="AO11" t="str"/>
-      <x:c r="AP11" t="str"/>
-      <x:c r="AQ11" t="str"/>
-      <x:c r="AR11" t="str"/>
-      <x:c r="AS11" t="str"/>
-      <x:c r="AT11" t="str"/>
-      <x:c r="AU11" t="str"/>
-      <x:c r="AV11" t="str"/>
-      <x:c r="AW11" t="str"/>
-      <x:c r="AX11" t="str"/>
+      <x:c r="I11" s="6" t="str"/>
+      <x:c r="J11" s="6" t="str"/>
+      <x:c r="K11" s="6" t="str"/>
+      <x:c r="L11" s="6" t="str"/>
+      <x:c r="M11" s="6" t="str"/>
+      <x:c r="N11" s="6" t="str"/>
+      <x:c r="O11" s="6" t="str"/>
+      <x:c r="P11" s="6" t="str"/>
+      <x:c r="Q11" s="7" t="str"/>
+      <x:c r="R11" s="7" t="str"/>
+      <x:c r="S11" s="7" t="str"/>
+      <x:c r="T11" s="7" t="str"/>
+      <x:c r="U11" s="7" t="str"/>
+      <x:c r="V11" s="7" t="str"/>
+      <x:c r="W11" s="7" t="str"/>
+      <x:c r="X11" s="6" t="str"/>
+      <x:c r="Y11" s="6" t="str"/>
+      <x:c r="Z11" s="6" t="str"/>
+      <x:c r="AA11" s="6" t="str"/>
+      <x:c r="AB11" s="6" t="str"/>
+      <x:c r="AC11" s="6" t="str"/>
+      <x:c r="AD11" s="6" t="str"/>
+      <x:c r="AE11" s="6" t="str"/>
+      <x:c r="AF11" s="6" t="str"/>
+      <x:c r="AG11" s="6" t="str"/>
+      <x:c r="AH11" s="6" t="str"/>
+      <x:c r="AI11" s="6" t="str"/>
+      <x:c r="AJ11" s="6" t="str"/>
+      <x:c r="AK11" s="6" t="str"/>
+      <x:c r="AL11" s="6" t="str"/>
+      <x:c r="AM11" s="6" t="str"/>
+      <x:c r="AN11" s="6" t="str"/>
+      <x:c r="AO11" s="6" t="str"/>
+      <x:c r="AP11" s="6" t="str"/>
+      <x:c r="AQ11" s="6" t="str"/>
+      <x:c r="AR11" s="6" t="str"/>
+      <x:c r="AS11" s="6" t="str"/>
+      <x:c r="AT11" s="6" t="str"/>
+      <x:c r="AU11" s="6" t="str"/>
+      <x:c r="AV11" s="6" t="str"/>
+      <x:c r="AW11" s="6" t="str"/>
+      <x:c r="AX11" s="6" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>2.3</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>아키텍처 문서 작성</x:v>
+        <x:v>React Native Expo TypeScript 선택</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D12" s="8" t="str">
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>2026-05-22</x:v>
+        <x:v>2026-05-19</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>2026-05-24</x:v>
+        <x:v>2026-05-20</x:v>
       </x:c>
       <x:c r="G12" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H12" t="n">
         <x:v>100</x:v>
@@ -1179,12 +1192,12 @@
       <x:c r="N12" t="str"/>
       <x:c r="O12" t="str"/>
       <x:c r="P12" t="str"/>
-      <x:c r="Q12" t="str"/>
-      <x:c r="R12" t="str"/>
+      <x:c r="Q12" s="9" t="str"/>
+      <x:c r="R12" s="9" t="str"/>
       <x:c r="S12" t="str"/>
-      <x:c r="T12" s="9" t="str"/>
-      <x:c r="U12" s="9" t="str"/>
-      <x:c r="V12" s="9" t="str"/>
+      <x:c r="T12" t="str"/>
+      <x:c r="U12" t="str"/>
+      <x:c r="V12" t="str"/>
       <x:c r="W12" t="str"/>
       <x:c r="X12" t="str"/>
       <x:c r="Y12" t="str"/>
@@ -1216,25 +1229,25 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>2.4</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>GitHub Pages 발표 페이지 구성</x:v>
+        <x:v>ADR 작성</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>윤서호</x:v>
+        <x:v>정원식</x:v>
       </x:c>
       <x:c r="D13" s="8" t="str">
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>2026-05-24</x:v>
+        <x:v>2026-05-20</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>2026-05-25</x:v>
+        <x:v>2026-05-22</x:v>
       </x:c>
       <x:c r="G13" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H13" t="n">
         <x:v>100</x:v>
@@ -1248,12 +1261,12 @@
       <x:c r="O13" t="str"/>
       <x:c r="P13" t="str"/>
       <x:c r="Q13" t="str"/>
-      <x:c r="R13" t="str"/>
-      <x:c r="S13" t="str"/>
-      <x:c r="T13" t="str"/>
+      <x:c r="R13" s="9" t="str"/>
+      <x:c r="S13" s="9" t="str"/>
+      <x:c r="T13" s="9" t="str"/>
       <x:c r="U13" t="str"/>
-      <x:c r="V13" s="9" t="str"/>
-      <x:c r="W13" s="9" t="str"/>
+      <x:c r="V13" t="str"/>
+      <x:c r="W13" t="str"/>
       <x:c r="X13" t="str"/>
       <x:c r="Y13" t="str"/>
       <x:c r="Z13" t="str"/>
@@ -1283,97 +1296,97 @@
       <x:c r="AX13" t="str"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="6" t="str">
+      <x:c r="A14" t="str">
+        <x:v>2.3</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Mermaid 아키텍처 문서 작성</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D14" s="8" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>2026-05-22</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>2026-05-24</x:v>
+      </x:c>
+      <x:c r="G14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B14" s="6" t="str">
-        <x:v>핵심 입력 기능</x:v>
-      </x:c>
-      <x:c r="C14" s="6" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="D14" s="6" t="str">
-        <x:v>In Progress</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="str">
-        <x:v>2026-05-26</x:v>
-      </x:c>
-      <x:c r="F14" s="6" t="str">
-        <x:v>2026-06-01</x:v>
-      </x:c>
-      <x:c r="G14" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H14" s="6" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="I14" s="6" t="str"/>
-      <x:c r="J14" s="6" t="str"/>
-      <x:c r="K14" s="6" t="str"/>
-      <x:c r="L14" s="6" t="str"/>
-      <x:c r="M14" s="6" t="str"/>
-      <x:c r="N14" s="6" t="str"/>
-      <x:c r="O14" s="6" t="str"/>
-      <x:c r="P14" s="6" t="str"/>
-      <x:c r="Q14" s="6" t="str"/>
-      <x:c r="R14" s="6" t="str"/>
-      <x:c r="S14" s="6" t="str"/>
-      <x:c r="T14" s="6" t="str"/>
-      <x:c r="U14" s="6" t="str"/>
-      <x:c r="V14" s="6" t="str"/>
-      <x:c r="W14" s="6" t="str"/>
-      <x:c r="X14" s="10" t="str"/>
-      <x:c r="Y14" s="10" t="str"/>
-      <x:c r="Z14" s="10" t="str"/>
-      <x:c r="AA14" s="10" t="str"/>
-      <x:c r="AB14" s="10" t="str"/>
-      <x:c r="AC14" s="10" t="str"/>
-      <x:c r="AD14" s="10" t="str"/>
-      <x:c r="AE14" s="6" t="str"/>
-      <x:c r="AF14" s="6" t="str"/>
-      <x:c r="AG14" s="6" t="str"/>
-      <x:c r="AH14" s="6" t="str"/>
-      <x:c r="AI14" s="6" t="str"/>
-      <x:c r="AJ14" s="6" t="str"/>
-      <x:c r="AK14" s="6" t="str"/>
-      <x:c r="AL14" s="6" t="str"/>
-      <x:c r="AM14" s="6" t="str"/>
-      <x:c r="AN14" s="6" t="str"/>
-      <x:c r="AO14" s="6" t="str"/>
-      <x:c r="AP14" s="6" t="str"/>
-      <x:c r="AQ14" s="6" t="str"/>
-      <x:c r="AR14" s="6" t="str"/>
-      <x:c r="AS14" s="6" t="str"/>
-      <x:c r="AT14" s="6" t="str"/>
-      <x:c r="AU14" s="6" t="str"/>
-      <x:c r="AV14" s="6" t="str"/>
-      <x:c r="AW14" s="6" t="str"/>
-      <x:c r="AX14" s="6" t="str"/>
+      <x:c r="H14" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I14" t="str"/>
+      <x:c r="J14" t="str"/>
+      <x:c r="K14" t="str"/>
+      <x:c r="L14" t="str"/>
+      <x:c r="M14" t="str"/>
+      <x:c r="N14" t="str"/>
+      <x:c r="O14" t="str"/>
+      <x:c r="P14" t="str"/>
+      <x:c r="Q14" t="str"/>
+      <x:c r="R14" t="str"/>
+      <x:c r="S14" t="str"/>
+      <x:c r="T14" s="9" t="str"/>
+      <x:c r="U14" s="9" t="str"/>
+      <x:c r="V14" s="9" t="str"/>
+      <x:c r="W14" t="str"/>
+      <x:c r="X14" t="str"/>
+      <x:c r="Y14" t="str"/>
+      <x:c r="Z14" t="str"/>
+      <x:c r="AA14" t="str"/>
+      <x:c r="AB14" t="str"/>
+      <x:c r="AC14" t="str"/>
+      <x:c r="AD14" t="str"/>
+      <x:c r="AE14" t="str"/>
+      <x:c r="AF14" t="str"/>
+      <x:c r="AG14" t="str"/>
+      <x:c r="AH14" t="str"/>
+      <x:c r="AI14" t="str"/>
+      <x:c r="AJ14" t="str"/>
+      <x:c r="AK14" t="str"/>
+      <x:c r="AL14" t="str"/>
+      <x:c r="AM14" t="str"/>
+      <x:c r="AN14" t="str"/>
+      <x:c r="AO14" t="str"/>
+      <x:c r="AP14" t="str"/>
+      <x:c r="AQ14" t="str"/>
+      <x:c r="AR14" t="str"/>
+      <x:c r="AS14" t="str"/>
+      <x:c r="AT14" t="str"/>
+      <x:c r="AU14" t="str"/>
+      <x:c r="AV14" t="str"/>
+      <x:c r="AW14" t="str"/>
+      <x:c r="AX14" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>3.1</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>컨디션 입력 화면</x:v>
+        <x:v>GitHub Pages 발표 페이지 구성</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D15" s="11" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D15" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>2026-05-26</x:v>
+        <x:v>2026-05-24</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>2026-05-29</x:v>
+        <x:v>2026-05-25</x:v>
       </x:c>
       <x:c r="G15" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H15" t="n">
-        <x:v>45</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I15" t="str"/>
       <x:c r="J15" t="str"/>
@@ -1388,12 +1401,12 @@
       <x:c r="S15" t="str"/>
       <x:c r="T15" t="str"/>
       <x:c r="U15" t="str"/>
-      <x:c r="V15" t="str"/>
-      <x:c r="W15" t="str"/>
-      <x:c r="X15" s="12" t="str"/>
-      <x:c r="Y15" s="12" t="str"/>
-      <x:c r="Z15" s="12" t="str"/>
-      <x:c r="AA15" s="12" t="str"/>
+      <x:c r="V15" s="9" t="str"/>
+      <x:c r="W15" s="9" t="str"/>
+      <x:c r="X15" t="str"/>
+      <x:c r="Y15" t="str"/>
+      <x:c r="Z15" t="str"/>
+      <x:c r="AA15" t="str"/>
       <x:c r="AB15" t="str"/>
       <x:c r="AC15" t="str"/>
       <x:c r="AD15" t="str"/>
@@ -1419,233 +1432,233 @@
       <x:c r="AX15" t="str"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>3.2</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>할 일 등록 화면</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>2026-05-29</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>2026-06-01</x:v>
-      </x:c>
-      <x:c r="G16" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" t="str"/>
-      <x:c r="J16" t="str"/>
-      <x:c r="K16" t="str"/>
-      <x:c r="L16" t="str"/>
-      <x:c r="M16" t="str"/>
-      <x:c r="N16" t="str"/>
-      <x:c r="O16" t="str"/>
-      <x:c r="P16" t="str"/>
-      <x:c r="Q16" t="str"/>
-      <x:c r="R16" t="str"/>
-      <x:c r="S16" t="str"/>
-      <x:c r="T16" t="str"/>
-      <x:c r="U16" t="str"/>
-      <x:c r="V16" t="str"/>
-      <x:c r="W16" t="str"/>
-      <x:c r="X16" t="str"/>
-      <x:c r="Y16" t="str"/>
-      <x:c r="Z16" t="str"/>
-      <x:c r="AA16" s="5" t="str"/>
-      <x:c r="AB16" s="5" t="str"/>
-      <x:c r="AC16" s="5" t="str"/>
-      <x:c r="AD16" s="5" t="str"/>
-      <x:c r="AE16" t="str"/>
-      <x:c r="AF16" t="str"/>
-      <x:c r="AG16" t="str"/>
-      <x:c r="AH16" t="str"/>
-      <x:c r="AI16" t="str"/>
-      <x:c r="AJ16" t="str"/>
-      <x:c r="AK16" t="str"/>
-      <x:c r="AL16" t="str"/>
-      <x:c r="AM16" t="str"/>
-      <x:c r="AN16" t="str"/>
-      <x:c r="AO16" t="str"/>
-      <x:c r="AP16" t="str"/>
-      <x:c r="AQ16" t="str"/>
-      <x:c r="AR16" t="str"/>
-      <x:c r="AS16" t="str"/>
-      <x:c r="AT16" t="str"/>
-      <x:c r="AU16" t="str"/>
-      <x:c r="AV16" t="str"/>
-      <x:c r="AW16" t="str"/>
-      <x:c r="AX16" t="str"/>
+      <x:c r="A16" s="11" t="str">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>개발 환경 점검</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
+        <x:v>Milestone</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="str">
+        <x:v>2026-05-25</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="str">
+        <x:v>2026-05-25</x:v>
+      </x:c>
+      <x:c r="G16" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="str"/>
+      <x:c r="J16" s="11" t="str"/>
+      <x:c r="K16" s="11" t="str"/>
+      <x:c r="L16" s="11" t="str"/>
+      <x:c r="M16" s="11" t="str"/>
+      <x:c r="N16" s="11" t="str"/>
+      <x:c r="O16" s="11" t="str"/>
+      <x:c r="P16" s="11" t="str"/>
+      <x:c r="Q16" s="11" t="str"/>
+      <x:c r="R16" s="11" t="str"/>
+      <x:c r="S16" s="11" t="str"/>
+      <x:c r="T16" s="11" t="str"/>
+      <x:c r="U16" s="11" t="str"/>
+      <x:c r="V16" s="11" t="str"/>
+      <x:c r="W16" s="12" t="str"/>
+      <x:c r="X16" s="11" t="str"/>
+      <x:c r="Y16" s="11" t="str"/>
+      <x:c r="Z16" s="11" t="str"/>
+      <x:c r="AA16" s="11" t="str"/>
+      <x:c r="AB16" s="11" t="str"/>
+      <x:c r="AC16" s="11" t="str"/>
+      <x:c r="AD16" s="11" t="str"/>
+      <x:c r="AE16" s="11" t="str"/>
+      <x:c r="AF16" s="11" t="str"/>
+      <x:c r="AG16" s="11" t="str"/>
+      <x:c r="AH16" s="11" t="str"/>
+      <x:c r="AI16" s="11" t="str"/>
+      <x:c r="AJ16" s="11" t="str"/>
+      <x:c r="AK16" s="11" t="str"/>
+      <x:c r="AL16" s="11" t="str"/>
+      <x:c r="AM16" s="11" t="str"/>
+      <x:c r="AN16" s="11" t="str"/>
+      <x:c r="AO16" s="11" t="str"/>
+      <x:c r="AP16" s="11" t="str"/>
+      <x:c r="AQ16" s="11" t="str"/>
+      <x:c r="AR16" s="11" t="str"/>
+      <x:c r="AS16" s="11" t="str"/>
+      <x:c r="AT16" s="11" t="str"/>
+      <x:c r="AU16" s="11" t="str"/>
+      <x:c r="AV16" s="11" t="str"/>
+      <x:c r="AW16" s="11" t="str"/>
+      <x:c r="AX16" s="11" t="str"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>3.3</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>입력값 검증 규칙</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>2026-06-01</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>2026-06-01</x:v>
-      </x:c>
-      <x:c r="G17" t="n">
+      <x:c r="A17" s="6" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>Energy Budget MVP 앱 구현</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>2026-05-26</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I17" s="6" t="str"/>
+      <x:c r="J17" s="6" t="str"/>
+      <x:c r="K17" s="6" t="str"/>
+      <x:c r="L17" s="6" t="str"/>
+      <x:c r="M17" s="6" t="str"/>
+      <x:c r="N17" s="6" t="str"/>
+      <x:c r="O17" s="6" t="str"/>
+      <x:c r="P17" s="6" t="str"/>
+      <x:c r="Q17" s="6" t="str"/>
+      <x:c r="R17" s="6" t="str"/>
+      <x:c r="S17" s="6" t="str"/>
+      <x:c r="T17" s="6" t="str"/>
+      <x:c r="U17" s="6" t="str"/>
+      <x:c r="V17" s="6" t="str"/>
+      <x:c r="W17" s="6" t="str"/>
+      <x:c r="X17" s="7" t="str"/>
+      <x:c r="Y17" s="7" t="str"/>
+      <x:c r="Z17" s="7" t="str"/>
+      <x:c r="AA17" s="6" t="str"/>
+      <x:c r="AB17" s="6" t="str"/>
+      <x:c r="AC17" s="6" t="str"/>
+      <x:c r="AD17" s="6" t="str"/>
+      <x:c r="AE17" s="6" t="str"/>
+      <x:c r="AF17" s="6" t="str"/>
+      <x:c r="AG17" s="6" t="str"/>
+      <x:c r="AH17" s="6" t="str"/>
+      <x:c r="AI17" s="6" t="str"/>
+      <x:c r="AJ17" s="6" t="str"/>
+      <x:c r="AK17" s="6" t="str"/>
+      <x:c r="AL17" s="6" t="str"/>
+      <x:c r="AM17" s="6" t="str"/>
+      <x:c r="AN17" s="6" t="str"/>
+      <x:c r="AO17" s="6" t="str"/>
+      <x:c r="AP17" s="6" t="str"/>
+      <x:c r="AQ17" s="6" t="str"/>
+      <x:c r="AR17" s="6" t="str"/>
+      <x:c r="AS17" s="6" t="str"/>
+      <x:c r="AT17" s="6" t="str"/>
+      <x:c r="AU17" s="6" t="str"/>
+      <x:c r="AV17" s="6" t="str"/>
+      <x:c r="AW17" s="6" t="str"/>
+      <x:c r="AX17" s="6" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>3.1</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>에너지 예산 계산 규칙 구현</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>2026-05-26</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>2026-05-26</x:v>
+      </x:c>
+      <x:c r="G18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I17" t="str"/>
-      <x:c r="J17" t="str"/>
-      <x:c r="K17" t="str"/>
-      <x:c r="L17" t="str"/>
-      <x:c r="M17" t="str"/>
-      <x:c r="N17" t="str"/>
-      <x:c r="O17" t="str"/>
-      <x:c r="P17" t="str"/>
-      <x:c r="Q17" t="str"/>
-      <x:c r="R17" t="str"/>
-      <x:c r="S17" t="str"/>
-      <x:c r="T17" t="str"/>
-      <x:c r="U17" t="str"/>
-      <x:c r="V17" t="str"/>
-      <x:c r="W17" t="str"/>
-      <x:c r="X17" t="str"/>
-      <x:c r="Y17" t="str"/>
-      <x:c r="Z17" t="str"/>
-      <x:c r="AA17" t="str"/>
-      <x:c r="AB17" t="str"/>
-      <x:c r="AC17" t="str"/>
-      <x:c r="AD17" s="5" t="str"/>
-      <x:c r="AE17" t="str"/>
-      <x:c r="AF17" t="str"/>
-      <x:c r="AG17" t="str"/>
-      <x:c r="AH17" t="str"/>
-      <x:c r="AI17" t="str"/>
-      <x:c r="AJ17" t="str"/>
-      <x:c r="AK17" t="str"/>
-      <x:c r="AL17" t="str"/>
-      <x:c r="AM17" t="str"/>
-      <x:c r="AN17" t="str"/>
-      <x:c r="AO17" t="str"/>
-      <x:c r="AP17" t="str"/>
-      <x:c r="AQ17" t="str"/>
-      <x:c r="AR17" t="str"/>
-      <x:c r="AS17" t="str"/>
-      <x:c r="AT17" t="str"/>
-      <x:c r="AU17" t="str"/>
-      <x:c r="AV17" t="str"/>
-      <x:c r="AW17" t="str"/>
-      <x:c r="AX17" t="str"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="6" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>에너지 예산 계산</x:v>
-      </x:c>
-      <x:c r="C18" s="6" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="D18" s="6" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E18" s="6" t="str">
-        <x:v>2026-06-02</x:v>
-      </x:c>
-      <x:c r="F18" s="6" t="str">
-        <x:v>2026-06-08</x:v>
-      </x:c>
-      <x:c r="G18" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H18" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I18" s="6" t="str"/>
-      <x:c r="J18" s="6" t="str"/>
-      <x:c r="K18" s="6" t="str"/>
-      <x:c r="L18" s="6" t="str"/>
-      <x:c r="M18" s="6" t="str"/>
-      <x:c r="N18" s="6" t="str"/>
-      <x:c r="O18" s="6" t="str"/>
-      <x:c r="P18" s="6" t="str"/>
-      <x:c r="Q18" s="6" t="str"/>
-      <x:c r="R18" s="6" t="str"/>
-      <x:c r="S18" s="6" t="str"/>
-      <x:c r="T18" s="6" t="str"/>
-      <x:c r="U18" s="6" t="str"/>
-      <x:c r="V18" s="6" t="str"/>
-      <x:c r="W18" s="6" t="str"/>
-      <x:c r="X18" s="6" t="str"/>
-      <x:c r="Y18" s="6" t="str"/>
-      <x:c r="Z18" s="6" t="str"/>
-      <x:c r="AA18" s="6" t="str"/>
-      <x:c r="AB18" s="6" t="str"/>
-      <x:c r="AC18" s="6" t="str"/>
-      <x:c r="AD18" s="6" t="str"/>
-      <x:c r="AE18" s="6" t="str"/>
-      <x:c r="AF18" s="6" t="str"/>
-      <x:c r="AG18" s="6" t="str"/>
-      <x:c r="AH18" s="6" t="str"/>
-      <x:c r="AI18" s="6" t="str"/>
-      <x:c r="AJ18" s="6" t="str"/>
-      <x:c r="AK18" s="6" t="str"/>
-      <x:c r="AL18" s="6" t="str"/>
-      <x:c r="AM18" s="6" t="str"/>
-      <x:c r="AN18" s="6" t="str"/>
-      <x:c r="AO18" s="6" t="str"/>
-      <x:c r="AP18" s="6" t="str"/>
-      <x:c r="AQ18" s="6" t="str"/>
-      <x:c r="AR18" s="6" t="str"/>
-      <x:c r="AS18" s="6" t="str"/>
-      <x:c r="AT18" s="6" t="str"/>
-      <x:c r="AU18" s="6" t="str"/>
-      <x:c r="AV18" s="6" t="str"/>
-      <x:c r="AW18" s="6" t="str"/>
-      <x:c r="AX18" s="6" t="str"/>
+      <x:c r="H18" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I18" t="str"/>
+      <x:c r="J18" t="str"/>
+      <x:c r="K18" t="str"/>
+      <x:c r="L18" t="str"/>
+      <x:c r="M18" t="str"/>
+      <x:c r="N18" t="str"/>
+      <x:c r="O18" t="str"/>
+      <x:c r="P18" t="str"/>
+      <x:c r="Q18" t="str"/>
+      <x:c r="R18" t="str"/>
+      <x:c r="S18" t="str"/>
+      <x:c r="T18" t="str"/>
+      <x:c r="U18" t="str"/>
+      <x:c r="V18" t="str"/>
+      <x:c r="W18" t="str"/>
+      <x:c r="X18" s="9" t="str"/>
+      <x:c r="Y18" t="str"/>
+      <x:c r="Z18" t="str"/>
+      <x:c r="AA18" t="str"/>
+      <x:c r="AB18" t="str"/>
+      <x:c r="AC18" t="str"/>
+      <x:c r="AD18" t="str"/>
+      <x:c r="AE18" t="str"/>
+      <x:c r="AF18" t="str"/>
+      <x:c r="AG18" t="str"/>
+      <x:c r="AH18" t="str"/>
+      <x:c r="AI18" t="str"/>
+      <x:c r="AJ18" t="str"/>
+      <x:c r="AK18" t="str"/>
+      <x:c r="AL18" t="str"/>
+      <x:c r="AM18" t="str"/>
+      <x:c r="AN18" t="str"/>
+      <x:c r="AO18" t="str"/>
+      <x:c r="AP18" t="str"/>
+      <x:c r="AQ18" t="str"/>
+      <x:c r="AR18" t="str"/>
+      <x:c r="AS18" t="str"/>
+      <x:c r="AT18" t="str"/>
+      <x:c r="AU18" t="str"/>
+      <x:c r="AV18" t="str"/>
+      <x:c r="AW18" t="str"/>
+      <x:c r="AX18" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>4.1</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>에너지 계산 규칙</x:v>
+        <x:v>컨디션 입력 UI 구현</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D19" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>2026-06-02</x:v>
+        <x:v>2026-05-26</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>2026-06-04</x:v>
+        <x:v>2026-05-27</x:v>
       </x:c>
       <x:c r="G19" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H19" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I19" t="str"/>
       <x:c r="J19" t="str"/>
@@ -1662,16 +1675,16 @@
       <x:c r="U19" t="str"/>
       <x:c r="V19" t="str"/>
       <x:c r="W19" t="str"/>
-      <x:c r="X19" t="str"/>
-      <x:c r="Y19" t="str"/>
+      <x:c r="X19" s="9" t="str"/>
+      <x:c r="Y19" s="9" t="str"/>
       <x:c r="Z19" t="str"/>
       <x:c r="AA19" t="str"/>
       <x:c r="AB19" t="str"/>
       <x:c r="AC19" t="str"/>
       <x:c r="AD19" t="str"/>
-      <x:c r="AE19" s="5" t="str"/>
-      <x:c r="AF19" s="5" t="str"/>
-      <x:c r="AG19" s="5" t="str"/>
+      <x:c r="AE19" t="str"/>
+      <x:c r="AF19" t="str"/>
+      <x:c r="AG19" t="str"/>
       <x:c r="AH19" t="str"/>
       <x:c r="AI19" t="str"/>
       <x:c r="AJ19" t="str"/>
@@ -1692,28 +1705,28 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>4.2</x:v>
+        <x:v>3.3</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>과부하 판단 기능</x:v>
+        <x:v>할 일 추가 UI 구현</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>2026-06-04</x:v>
+        <x:v>2026-05-27</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>2026-06-06</x:v>
+        <x:v>2026-05-27</x:v>
       </x:c>
       <x:c r="G20" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H20" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I20" t="str"/>
       <x:c r="J20" t="str"/>
@@ -1731,7 +1744,7 @@
       <x:c r="V20" t="str"/>
       <x:c r="W20" t="str"/>
       <x:c r="X20" t="str"/>
-      <x:c r="Y20" t="str"/>
+      <x:c r="Y20" s="9" t="str"/>
       <x:c r="Z20" t="str"/>
       <x:c r="AA20" t="str"/>
       <x:c r="AB20" t="str"/>
@@ -1739,9 +1752,9 @@
       <x:c r="AD20" t="str"/>
       <x:c r="AE20" t="str"/>
       <x:c r="AF20" t="str"/>
-      <x:c r="AG20" s="5" t="str"/>
-      <x:c r="AH20" s="5" t="str"/>
-      <x:c r="AI20" s="5" t="str"/>
+      <x:c r="AG20" t="str"/>
+      <x:c r="AH20" t="str"/>
+      <x:c r="AI20" t="str"/>
       <x:c r="AJ20" t="str"/>
       <x:c r="AK20" t="str"/>
       <x:c r="AL20" t="str"/>
@@ -1760,28 +1773,28 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>4.3</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>추천 결과 화면</x:v>
+        <x:v>추천 및 미루기 목록 구현</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E21" t="str">
-        <x:v>2026-06-06</x:v>
+        <x:v>2026-05-27</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="G21" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H21" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I21" t="str"/>
       <x:c r="J21" t="str"/>
@@ -1799,8 +1812,8 @@
       <x:c r="V21" t="str"/>
       <x:c r="W21" t="str"/>
       <x:c r="X21" t="str"/>
-      <x:c r="Y21" t="str"/>
-      <x:c r="Z21" t="str"/>
+      <x:c r="Y21" s="9" t="str"/>
+      <x:c r="Z21" s="9" t="str"/>
       <x:c r="AA21" t="str"/>
       <x:c r="AB21" t="str"/>
       <x:c r="AC21" t="str"/>
@@ -1809,9 +1822,9 @@
       <x:c r="AF21" t="str"/>
       <x:c r="AG21" t="str"/>
       <x:c r="AH21" t="str"/>
-      <x:c r="AI21" s="5" t="str"/>
-      <x:c r="AJ21" s="5" t="str"/>
-      <x:c r="AK21" s="5" t="str"/>
+      <x:c r="AI21" t="str"/>
+      <x:c r="AJ21" t="str"/>
+      <x:c r="AK21" t="str"/>
       <x:c r="AL21" t="str"/>
       <x:c r="AM21" t="str"/>
       <x:c r="AN21" t="str"/>
@@ -1827,97 +1840,97 @@
       <x:c r="AX21" t="str"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="6" t="str">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B22" s="6" t="str">
-        <x:v>기록과 리포트</x:v>
-      </x:c>
-      <x:c r="C22" s="6" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="D22" s="6" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E22" s="6" t="str">
-        <x:v>2026-06-09</x:v>
-      </x:c>
-      <x:c r="F22" s="6" t="str">
-        <x:v>2026-06-15</x:v>
-      </x:c>
-      <x:c r="G22" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H22" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I22" s="6" t="str"/>
-      <x:c r="J22" s="6" t="str"/>
-      <x:c r="K22" s="6" t="str"/>
-      <x:c r="L22" s="6" t="str"/>
-      <x:c r="M22" s="6" t="str"/>
-      <x:c r="N22" s="6" t="str"/>
-      <x:c r="O22" s="6" t="str"/>
-      <x:c r="P22" s="6" t="str"/>
-      <x:c r="Q22" s="6" t="str"/>
-      <x:c r="R22" s="6" t="str"/>
-      <x:c r="S22" s="6" t="str"/>
-      <x:c r="T22" s="6" t="str"/>
-      <x:c r="U22" s="6" t="str"/>
-      <x:c r="V22" s="6" t="str"/>
-      <x:c r="W22" s="6" t="str"/>
-      <x:c r="X22" s="6" t="str"/>
-      <x:c r="Y22" s="6" t="str"/>
-      <x:c r="Z22" s="6" t="str"/>
-      <x:c r="AA22" s="6" t="str"/>
-      <x:c r="AB22" s="6" t="str"/>
-      <x:c r="AC22" s="6" t="str"/>
-      <x:c r="AD22" s="6" t="str"/>
-      <x:c r="AE22" s="6" t="str"/>
-      <x:c r="AF22" s="6" t="str"/>
-      <x:c r="AG22" s="6" t="str"/>
-      <x:c r="AH22" s="6" t="str"/>
-      <x:c r="AI22" s="6" t="str"/>
-      <x:c r="AJ22" s="6" t="str"/>
-      <x:c r="AK22" s="6" t="str"/>
-      <x:c r="AL22" s="6" t="str"/>
-      <x:c r="AM22" s="6" t="str"/>
-      <x:c r="AN22" s="6" t="str"/>
-      <x:c r="AO22" s="6" t="str"/>
-      <x:c r="AP22" s="6" t="str"/>
-      <x:c r="AQ22" s="6" t="str"/>
-      <x:c r="AR22" s="6" t="str"/>
-      <x:c r="AS22" s="6" t="str"/>
-      <x:c r="AT22" s="6" t="str"/>
-      <x:c r="AU22" s="6" t="str"/>
-      <x:c r="AV22" s="6" t="str"/>
-      <x:c r="AW22" s="6" t="str"/>
-      <x:c r="AX22" s="6" t="str"/>
+      <x:c r="A22" t="str">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>실행 배치 파일 작성</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D22" s="8" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H22" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I22" t="str"/>
+      <x:c r="J22" t="str"/>
+      <x:c r="K22" t="str"/>
+      <x:c r="L22" t="str"/>
+      <x:c r="M22" t="str"/>
+      <x:c r="N22" t="str"/>
+      <x:c r="O22" t="str"/>
+      <x:c r="P22" t="str"/>
+      <x:c r="Q22" t="str"/>
+      <x:c r="R22" t="str"/>
+      <x:c r="S22" t="str"/>
+      <x:c r="T22" t="str"/>
+      <x:c r="U22" t="str"/>
+      <x:c r="V22" t="str"/>
+      <x:c r="W22" t="str"/>
+      <x:c r="X22" t="str"/>
+      <x:c r="Y22" t="str"/>
+      <x:c r="Z22" s="9" t="str"/>
+      <x:c r="AA22" t="str"/>
+      <x:c r="AB22" t="str"/>
+      <x:c r="AC22" t="str"/>
+      <x:c r="AD22" t="str"/>
+      <x:c r="AE22" t="str"/>
+      <x:c r="AF22" t="str"/>
+      <x:c r="AG22" t="str"/>
+      <x:c r="AH22" t="str"/>
+      <x:c r="AI22" t="str"/>
+      <x:c r="AJ22" t="str"/>
+      <x:c r="AK22" t="str"/>
+      <x:c r="AL22" t="str"/>
+      <x:c r="AM22" t="str"/>
+      <x:c r="AN22" t="str"/>
+      <x:c r="AO22" t="str"/>
+      <x:c r="AP22" t="str"/>
+      <x:c r="AQ22" t="str"/>
+      <x:c r="AR22" t="str"/>
+      <x:c r="AS22" t="str"/>
+      <x:c r="AT22" t="str"/>
+      <x:c r="AU22" t="str"/>
+      <x:c r="AV22" t="str"/>
+      <x:c r="AW22" t="str"/>
+      <x:c r="AX22" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>5.1</x:v>
+        <x:v>3.6</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>일일 계획 저장</x:v>
+        <x:v>TypeScript 및 Expo export 검증</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E23" t="str">
-        <x:v>2026-06-09</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>2026-06-11</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="G23" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H23" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I23" t="str"/>
       <x:c r="J23" t="str"/>
@@ -1936,7 +1949,7 @@
       <x:c r="W23" t="str"/>
       <x:c r="X23" t="str"/>
       <x:c r="Y23" t="str"/>
-      <x:c r="Z23" t="str"/>
+      <x:c r="Z23" s="9" t="str"/>
       <x:c r="AA23" t="str"/>
       <x:c r="AB23" t="str"/>
       <x:c r="AC23" t="str"/>
@@ -1948,9 +1961,9 @@
       <x:c r="AI23" t="str"/>
       <x:c r="AJ23" t="str"/>
       <x:c r="AK23" t="str"/>
-      <x:c r="AL23" s="5" t="str"/>
-      <x:c r="AM23" s="5" t="str"/>
-      <x:c r="AN23" s="5" t="str"/>
+      <x:c r="AL23" t="str"/>
+      <x:c r="AM23" t="str"/>
+      <x:c r="AN23" t="str"/>
       <x:c r="AO23" t="str"/>
       <x:c r="AP23" t="str"/>
       <x:c r="AQ23" t="str"/>
@@ -1963,233 +1976,233 @@
       <x:c r="AX23" t="str"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" t="str">
-        <x:v>5.2</x:v>
-      </x:c>
-      <x:c r="B24" t="str">
-        <x:v>완료 여부 체크</x:v>
-      </x:c>
-      <x:c r="C24" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D24" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E24" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-      <x:c r="F24" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-      <x:c r="G24" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I24" t="str"/>
-      <x:c r="J24" t="str"/>
-      <x:c r="K24" t="str"/>
-      <x:c r="L24" t="str"/>
-      <x:c r="M24" t="str"/>
-      <x:c r="N24" t="str"/>
-      <x:c r="O24" t="str"/>
-      <x:c r="P24" t="str"/>
-      <x:c r="Q24" t="str"/>
-      <x:c r="R24" t="str"/>
-      <x:c r="S24" t="str"/>
-      <x:c r="T24" t="str"/>
-      <x:c r="U24" t="str"/>
-      <x:c r="V24" t="str"/>
-      <x:c r="W24" t="str"/>
-      <x:c r="X24" t="str"/>
-      <x:c r="Y24" t="str"/>
-      <x:c r="Z24" t="str"/>
-      <x:c r="AA24" t="str"/>
-      <x:c r="AB24" t="str"/>
-      <x:c r="AC24" t="str"/>
-      <x:c r="AD24" t="str"/>
-      <x:c r="AE24" t="str"/>
-      <x:c r="AF24" t="str"/>
-      <x:c r="AG24" t="str"/>
-      <x:c r="AH24" t="str"/>
-      <x:c r="AI24" t="str"/>
-      <x:c r="AJ24" t="str"/>
-      <x:c r="AK24" t="str"/>
-      <x:c r="AL24" t="str"/>
-      <x:c r="AM24" t="str"/>
-      <x:c r="AN24" s="5" t="str"/>
-      <x:c r="AO24" s="5" t="str"/>
-      <x:c r="AP24" s="5" t="str"/>
-      <x:c r="AQ24" t="str"/>
-      <x:c r="AR24" t="str"/>
-      <x:c r="AS24" t="str"/>
-      <x:c r="AT24" t="str"/>
-      <x:c r="AU24" t="str"/>
-      <x:c r="AV24" t="str"/>
-      <x:c r="AW24" t="str"/>
-      <x:c r="AX24" t="str"/>
+      <x:c r="A24" s="11" t="str">
+        <x:v>3.7</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="str">
+        <x:v>MVP 구현 점검</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="str">
+        <x:v>Milestone</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="G24" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H24" s="11" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="str"/>
+      <x:c r="J24" s="11" t="str"/>
+      <x:c r="K24" s="11" t="str"/>
+      <x:c r="L24" s="11" t="str"/>
+      <x:c r="M24" s="11" t="str"/>
+      <x:c r="N24" s="11" t="str"/>
+      <x:c r="O24" s="11" t="str"/>
+      <x:c r="P24" s="11" t="str"/>
+      <x:c r="Q24" s="11" t="str"/>
+      <x:c r="R24" s="11" t="str"/>
+      <x:c r="S24" s="11" t="str"/>
+      <x:c r="T24" s="11" t="str"/>
+      <x:c r="U24" s="11" t="str"/>
+      <x:c r="V24" s="11" t="str"/>
+      <x:c r="W24" s="11" t="str"/>
+      <x:c r="X24" s="11" t="str"/>
+      <x:c r="Y24" s="11" t="str"/>
+      <x:c r="Z24" s="12" t="str"/>
+      <x:c r="AA24" s="11" t="str"/>
+      <x:c r="AB24" s="11" t="str"/>
+      <x:c r="AC24" s="11" t="str"/>
+      <x:c r="AD24" s="11" t="str"/>
+      <x:c r="AE24" s="11" t="str"/>
+      <x:c r="AF24" s="11" t="str"/>
+      <x:c r="AG24" s="11" t="str"/>
+      <x:c r="AH24" s="11" t="str"/>
+      <x:c r="AI24" s="11" t="str"/>
+      <x:c r="AJ24" s="11" t="str"/>
+      <x:c r="AK24" s="11" t="str"/>
+      <x:c r="AL24" s="11" t="str"/>
+      <x:c r="AM24" s="11" t="str"/>
+      <x:c r="AN24" s="11" t="str"/>
+      <x:c r="AO24" s="11" t="str"/>
+      <x:c r="AP24" s="11" t="str"/>
+      <x:c r="AQ24" s="11" t="str"/>
+      <x:c r="AR24" s="11" t="str"/>
+      <x:c r="AS24" s="11" t="str"/>
+      <x:c r="AT24" s="11" t="str"/>
+      <x:c r="AU24" s="11" t="str"/>
+      <x:c r="AV24" s="11" t="str"/>
+      <x:c r="AW24" s="11" t="str"/>
+      <x:c r="AX24" s="11" t="str"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" t="str">
-        <x:v>5.3</x:v>
-      </x:c>
-      <x:c r="B25" t="str">
-        <x:v>주간 에너지 리포트</x:v>
-      </x:c>
-      <x:c r="C25" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D25" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E25" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-      <x:c r="F25" t="str">
-        <x:v>2026-06-15</x:v>
-      </x:c>
-      <x:c r="G25" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I25" t="str"/>
-      <x:c r="J25" t="str"/>
-      <x:c r="K25" t="str"/>
-      <x:c r="L25" t="str"/>
-      <x:c r="M25" t="str"/>
-      <x:c r="N25" t="str"/>
-      <x:c r="O25" t="str"/>
-      <x:c r="P25" t="str"/>
-      <x:c r="Q25" t="str"/>
-      <x:c r="R25" t="str"/>
-      <x:c r="S25" t="str"/>
-      <x:c r="T25" t="str"/>
-      <x:c r="U25" t="str"/>
-      <x:c r="V25" t="str"/>
-      <x:c r="W25" t="str"/>
-      <x:c r="X25" t="str"/>
-      <x:c r="Y25" t="str"/>
-      <x:c r="Z25" t="str"/>
-      <x:c r="AA25" t="str"/>
-      <x:c r="AB25" t="str"/>
-      <x:c r="AC25" t="str"/>
-      <x:c r="AD25" t="str"/>
-      <x:c r="AE25" t="str"/>
-      <x:c r="AF25" t="str"/>
-      <x:c r="AG25" t="str"/>
-      <x:c r="AH25" t="str"/>
-      <x:c r="AI25" t="str"/>
-      <x:c r="AJ25" t="str"/>
-      <x:c r="AK25" t="str"/>
-      <x:c r="AL25" t="str"/>
-      <x:c r="AM25" t="str"/>
-      <x:c r="AN25" t="str"/>
-      <x:c r="AO25" t="str"/>
-      <x:c r="AP25" s="5" t="str"/>
-      <x:c r="AQ25" s="5" t="str"/>
-      <x:c r="AR25" s="5" t="str"/>
-      <x:c r="AS25" t="str"/>
-      <x:c r="AT25" t="str"/>
-      <x:c r="AU25" t="str"/>
-      <x:c r="AV25" t="str"/>
-      <x:c r="AW25" t="str"/>
-      <x:c r="AX25" t="str"/>
+      <x:c r="A25" s="6" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="str">
+        <x:v>발표 자료 및 포트폴리오</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="E25" s="6" t="str">
+        <x:v>2026-05-27</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="str">
+        <x:v>2026-05-31</x:v>
+      </x:c>
+      <x:c r="G25" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H25" s="6" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="I25" s="6" t="str"/>
+      <x:c r="J25" s="6" t="str"/>
+      <x:c r="K25" s="6" t="str"/>
+      <x:c r="L25" s="6" t="str"/>
+      <x:c r="M25" s="6" t="str"/>
+      <x:c r="N25" s="6" t="str"/>
+      <x:c r="O25" s="6" t="str"/>
+      <x:c r="P25" s="6" t="str"/>
+      <x:c r="Q25" s="6" t="str"/>
+      <x:c r="R25" s="6" t="str"/>
+      <x:c r="S25" s="6" t="str"/>
+      <x:c r="T25" s="6" t="str"/>
+      <x:c r="U25" s="6" t="str"/>
+      <x:c r="V25" s="6" t="str"/>
+      <x:c r="W25" s="6" t="str"/>
+      <x:c r="X25" s="6" t="str"/>
+      <x:c r="Y25" s="13" t="str"/>
+      <x:c r="Z25" s="13" t="str"/>
+      <x:c r="AA25" s="13" t="str"/>
+      <x:c r="AB25" s="13" t="str"/>
+      <x:c r="AC25" s="13" t="str"/>
+      <x:c r="AD25" s="6" t="str"/>
+      <x:c r="AE25" s="6" t="str"/>
+      <x:c r="AF25" s="6" t="str"/>
+      <x:c r="AG25" s="6" t="str"/>
+      <x:c r="AH25" s="6" t="str"/>
+      <x:c r="AI25" s="6" t="str"/>
+      <x:c r="AJ25" s="6" t="str"/>
+      <x:c r="AK25" s="6" t="str"/>
+      <x:c r="AL25" s="6" t="str"/>
+      <x:c r="AM25" s="6" t="str"/>
+      <x:c r="AN25" s="6" t="str"/>
+      <x:c r="AO25" s="6" t="str"/>
+      <x:c r="AP25" s="6" t="str"/>
+      <x:c r="AQ25" s="6" t="str"/>
+      <x:c r="AR25" s="6" t="str"/>
+      <x:c r="AS25" s="6" t="str"/>
+      <x:c r="AT25" s="6" t="str"/>
+      <x:c r="AU25" s="6" t="str"/>
+      <x:c r="AV25" s="6" t="str"/>
+      <x:c r="AW25" s="6" t="str"/>
+      <x:c r="AX25" s="6" t="str"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="6" t="str">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B26" s="6" t="str">
-        <x:v>테스트와 발표 준비</x:v>
-      </x:c>
-      <x:c r="C26" s="6" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="D26" s="6" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E26" s="6" t="str">
-        <x:v>2026-06-16</x:v>
-      </x:c>
-      <x:c r="F26" s="6" t="str">
-        <x:v>2026-06-22</x:v>
-      </x:c>
-      <x:c r="G26" s="6" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H26" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I26" s="6" t="str"/>
-      <x:c r="J26" s="6" t="str"/>
-      <x:c r="K26" s="6" t="str"/>
-      <x:c r="L26" s="6" t="str"/>
-      <x:c r="M26" s="6" t="str"/>
-      <x:c r="N26" s="6" t="str"/>
-      <x:c r="O26" s="6" t="str"/>
-      <x:c r="P26" s="6" t="str"/>
-      <x:c r="Q26" s="6" t="str"/>
-      <x:c r="R26" s="6" t="str"/>
-      <x:c r="S26" s="6" t="str"/>
-      <x:c r="T26" s="6" t="str"/>
-      <x:c r="U26" s="6" t="str"/>
-      <x:c r="V26" s="6" t="str"/>
-      <x:c r="W26" s="6" t="str"/>
-      <x:c r="X26" s="6" t="str"/>
-      <x:c r="Y26" s="6" t="str"/>
-      <x:c r="Z26" s="6" t="str"/>
-      <x:c r="AA26" s="6" t="str"/>
-      <x:c r="AB26" s="6" t="str"/>
-      <x:c r="AC26" s="6" t="str"/>
-      <x:c r="AD26" s="6" t="str"/>
-      <x:c r="AE26" s="6" t="str"/>
-      <x:c r="AF26" s="6" t="str"/>
-      <x:c r="AG26" s="6" t="str"/>
-      <x:c r="AH26" s="6" t="str"/>
-      <x:c r="AI26" s="6" t="str"/>
-      <x:c r="AJ26" s="6" t="str"/>
-      <x:c r="AK26" s="6" t="str"/>
-      <x:c r="AL26" s="6" t="str"/>
-      <x:c r="AM26" s="6" t="str"/>
-      <x:c r="AN26" s="6" t="str"/>
-      <x:c r="AO26" s="6" t="str"/>
-      <x:c r="AP26" s="6" t="str"/>
-      <x:c r="AQ26" s="6" t="str"/>
-      <x:c r="AR26" s="6" t="str"/>
-      <x:c r="AS26" s="6" t="str"/>
-      <x:c r="AT26" s="6" t="str"/>
-      <x:c r="AU26" s="6" t="str"/>
-      <x:c r="AV26" s="6" t="str"/>
-      <x:c r="AW26" s="6" t="str"/>
-      <x:c r="AX26" s="6" t="str"/>
+      <x:c r="A26" t="str">
+        <x:v>4.1</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>스타트업 스타일 발표 PDF 제작</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D26" s="8" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>2026-05-27</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="G26" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H26" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I26" t="str"/>
+      <x:c r="J26" t="str"/>
+      <x:c r="K26" t="str"/>
+      <x:c r="L26" t="str"/>
+      <x:c r="M26" t="str"/>
+      <x:c r="N26" t="str"/>
+      <x:c r="O26" t="str"/>
+      <x:c r="P26" t="str"/>
+      <x:c r="Q26" t="str"/>
+      <x:c r="R26" t="str"/>
+      <x:c r="S26" t="str"/>
+      <x:c r="T26" t="str"/>
+      <x:c r="U26" t="str"/>
+      <x:c r="V26" t="str"/>
+      <x:c r="W26" t="str"/>
+      <x:c r="X26" t="str"/>
+      <x:c r="Y26" s="9" t="str"/>
+      <x:c r="Z26" s="9" t="str"/>
+      <x:c r="AA26" t="str"/>
+      <x:c r="AB26" t="str"/>
+      <x:c r="AC26" t="str"/>
+      <x:c r="AD26" t="str"/>
+      <x:c r="AE26" t="str"/>
+      <x:c r="AF26" t="str"/>
+      <x:c r="AG26" t="str"/>
+      <x:c r="AH26" t="str"/>
+      <x:c r="AI26" t="str"/>
+      <x:c r="AJ26" t="str"/>
+      <x:c r="AK26" t="str"/>
+      <x:c r="AL26" t="str"/>
+      <x:c r="AM26" t="str"/>
+      <x:c r="AN26" t="str"/>
+      <x:c r="AO26" t="str"/>
+      <x:c r="AP26" t="str"/>
+      <x:c r="AQ26" t="str"/>
+      <x:c r="AR26" t="str"/>
+      <x:c r="AS26" t="str"/>
+      <x:c r="AT26" t="str"/>
+      <x:c r="AU26" t="str"/>
+      <x:c r="AV26" t="str"/>
+      <x:c r="AW26" t="str"/>
+      <x:c r="AX26" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>6.1</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>사용자 시나리오 테스트</x:v>
+        <x:v>앱 화면 캡처 기반 PDF 수정</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D27" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D27" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E27" t="str">
-        <x:v>2026-06-16</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="F27" t="str">
-        <x:v>2026-06-18</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="G27" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H27" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I27" t="str"/>
       <x:c r="J27" t="str"/>
@@ -2208,7 +2221,7 @@
       <x:c r="W27" t="str"/>
       <x:c r="X27" t="str"/>
       <x:c r="Y27" t="str"/>
-      <x:c r="Z27" t="str"/>
+      <x:c r="Z27" s="9" t="str"/>
       <x:c r="AA27" t="str"/>
       <x:c r="AB27" t="str"/>
       <x:c r="AC27" t="str"/>
@@ -2227,37 +2240,37 @@
       <x:c r="AP27" t="str"/>
       <x:c r="AQ27" t="str"/>
       <x:c r="AR27" t="str"/>
-      <x:c r="AS27" s="5" t="str"/>
-      <x:c r="AT27" s="5" t="str"/>
-      <x:c r="AU27" s="5" t="str"/>
+      <x:c r="AS27" t="str"/>
+      <x:c r="AT27" t="str"/>
+      <x:c r="AU27" t="str"/>
       <x:c r="AV27" t="str"/>
       <x:c r="AW27" t="str"/>
       <x:c r="AX27" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>6.2</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>README와 발표 대사 정리</x:v>
+        <x:v>2분 발표 대사 작성</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D28" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D28" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E28" t="str">
-        <x:v>2026-06-18</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="F28" t="str">
-        <x:v>2026-06-20</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="G28" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H28" t="n">
-        <x:v>0</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I28" t="str"/>
       <x:c r="J28" t="str"/>
@@ -2276,7 +2289,7 @@
       <x:c r="W28" t="str"/>
       <x:c r="X28" t="str"/>
       <x:c r="Y28" t="str"/>
-      <x:c r="Z28" t="str"/>
+      <x:c r="Z28" s="9" t="str"/>
       <x:c r="AA28" t="str"/>
       <x:c r="AB28" t="str"/>
       <x:c r="AC28" t="str"/>
@@ -2297,35 +2310,35 @@
       <x:c r="AR28" t="str"/>
       <x:c r="AS28" t="str"/>
       <x:c r="AT28" t="str"/>
-      <x:c r="AU28" s="5" t="str"/>
-      <x:c r="AV28" s="5" t="str"/>
-      <x:c r="AW28" s="5" t="str"/>
+      <x:c r="AU28" t="str"/>
+      <x:c r="AV28" t="str"/>
+      <x:c r="AW28" t="str"/>
       <x:c r="AX28" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
-        <x:v>6.3</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>최종 발표 자료 배포</x:v>
+        <x:v>WBS Gantt 엑셀 최신화</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
-      <x:c r="D29" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E29" t="str">
-        <x:v>2026-06-20</x:v>
+        <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>2026-06-22</x:v>
+        <x:v>2026-05-29</x:v>
       </x:c>
       <x:c r="G29" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H29" t="n">
-        <x:v>0</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I29" t="str"/>
       <x:c r="J29" t="str"/>
@@ -2344,8 +2357,8 @@
       <x:c r="W29" t="str"/>
       <x:c r="X29" t="str"/>
       <x:c r="Y29" t="str"/>
-      <x:c r="Z29" t="str"/>
-      <x:c r="AA29" t="str"/>
+      <x:c r="Z29" s="15" t="str"/>
+      <x:c r="AA29" s="15" t="str"/>
       <x:c r="AB29" t="str"/>
       <x:c r="AC29" t="str"/>
       <x:c r="AD29" t="str"/>
@@ -2367,8 +2380,756 @@
       <x:c r="AT29" t="str"/>
       <x:c r="AU29" t="str"/>
       <x:c r="AV29" t="str"/>
-      <x:c r="AW29" s="5" t="str"/>
-      <x:c r="AX29" s="5" t="str"/>
+      <x:c r="AW29" t="str"/>
+      <x:c r="AX29" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>GitHub Pages 배포 점검</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>2026-05-29</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>2026-05-31</x:v>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H30" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="I30" t="str"/>
+      <x:c r="J30" t="str"/>
+      <x:c r="K30" t="str"/>
+      <x:c r="L30" t="str"/>
+      <x:c r="M30" t="str"/>
+      <x:c r="N30" t="str"/>
+      <x:c r="O30" t="str"/>
+      <x:c r="P30" t="str"/>
+      <x:c r="Q30" t="str"/>
+      <x:c r="R30" t="str"/>
+      <x:c r="S30" t="str"/>
+      <x:c r="T30" t="str"/>
+      <x:c r="U30" t="str"/>
+      <x:c r="V30" t="str"/>
+      <x:c r="W30" t="str"/>
+      <x:c r="X30" t="str"/>
+      <x:c r="Y30" t="str"/>
+      <x:c r="Z30" t="str"/>
+      <x:c r="AA30" s="15" t="str"/>
+      <x:c r="AB30" s="15" t="str"/>
+      <x:c r="AC30" s="15" t="str"/>
+      <x:c r="AD30" t="str"/>
+      <x:c r="AE30" t="str"/>
+      <x:c r="AF30" t="str"/>
+      <x:c r="AG30" t="str"/>
+      <x:c r="AH30" t="str"/>
+      <x:c r="AI30" t="str"/>
+      <x:c r="AJ30" t="str"/>
+      <x:c r="AK30" t="str"/>
+      <x:c r="AL30" t="str"/>
+      <x:c r="AM30" t="str"/>
+      <x:c r="AN30" t="str"/>
+      <x:c r="AO30" t="str"/>
+      <x:c r="AP30" t="str"/>
+      <x:c r="AQ30" t="str"/>
+      <x:c r="AR30" t="str"/>
+      <x:c r="AS30" t="str"/>
+      <x:c r="AT30" t="str"/>
+      <x:c r="AU30" t="str"/>
+      <x:c r="AV30" t="str"/>
+      <x:c r="AW30" t="str"/>
+      <x:c r="AX30" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="6" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B31" s="6" t="str">
+        <x:v>추가 기능 개발</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D31" s="6" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E31" s="6" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="F31" s="6" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="G31" s="6" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H31" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="6" t="str"/>
+      <x:c r="J31" s="6" t="str"/>
+      <x:c r="K31" s="6" t="str"/>
+      <x:c r="L31" s="6" t="str"/>
+      <x:c r="M31" s="6" t="str"/>
+      <x:c r="N31" s="6" t="str"/>
+      <x:c r="O31" s="6" t="str"/>
+      <x:c r="P31" s="6" t="str"/>
+      <x:c r="Q31" s="6" t="str"/>
+      <x:c r="R31" s="6" t="str"/>
+      <x:c r="S31" s="6" t="str"/>
+      <x:c r="T31" s="6" t="str"/>
+      <x:c r="U31" s="6" t="str"/>
+      <x:c r="V31" s="6" t="str"/>
+      <x:c r="W31" s="6" t="str"/>
+      <x:c r="X31" s="6" t="str"/>
+      <x:c r="Y31" s="6" t="str"/>
+      <x:c r="Z31" s="6" t="str"/>
+      <x:c r="AA31" s="6" t="str"/>
+      <x:c r="AB31" s="6" t="str"/>
+      <x:c r="AC31" s="6" t="str"/>
+      <x:c r="AD31" s="6" t="str"/>
+      <x:c r="AE31" s="6" t="str"/>
+      <x:c r="AF31" s="6" t="str"/>
+      <x:c r="AG31" s="6" t="str"/>
+      <x:c r="AH31" s="6" t="str"/>
+      <x:c r="AI31" s="6" t="str"/>
+      <x:c r="AJ31" s="6" t="str"/>
+      <x:c r="AK31" s="6" t="str"/>
+      <x:c r="AL31" s="6" t="str"/>
+      <x:c r="AM31" s="6" t="str"/>
+      <x:c r="AN31" s="6" t="str"/>
+      <x:c r="AO31" s="6" t="str"/>
+      <x:c r="AP31" s="6" t="str"/>
+      <x:c r="AQ31" s="6" t="str"/>
+      <x:c r="AR31" s="6" t="str"/>
+      <x:c r="AS31" s="6" t="str"/>
+      <x:c r="AT31" s="6" t="str"/>
+      <x:c r="AU31" s="6" t="str"/>
+      <x:c r="AV31" s="6" t="str"/>
+      <x:c r="AW31" s="6" t="str"/>
+      <x:c r="AX31" s="6" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>5.1</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>일일 계획 저장 기능</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>2026-06-05</x:v>
+      </x:c>
+      <x:c r="G32" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" t="str"/>
+      <x:c r="J32" t="str"/>
+      <x:c r="K32" t="str"/>
+      <x:c r="L32" t="str"/>
+      <x:c r="M32" t="str"/>
+      <x:c r="N32" t="str"/>
+      <x:c r="O32" t="str"/>
+      <x:c r="P32" t="str"/>
+      <x:c r="Q32" t="str"/>
+      <x:c r="R32" t="str"/>
+      <x:c r="S32" t="str"/>
+      <x:c r="T32" t="str"/>
+      <x:c r="U32" t="str"/>
+      <x:c r="V32" t="str"/>
+      <x:c r="W32" t="str"/>
+      <x:c r="X32" t="str"/>
+      <x:c r="Y32" t="str"/>
+      <x:c r="Z32" t="str"/>
+      <x:c r="AA32" t="str"/>
+      <x:c r="AB32" t="str"/>
+      <x:c r="AC32" t="str"/>
+      <x:c r="AD32" t="str"/>
+      <x:c r="AE32" s="5" t="str"/>
+      <x:c r="AF32" s="5" t="str"/>
+      <x:c r="AG32" s="5" t="str"/>
+      <x:c r="AH32" s="5" t="str"/>
+      <x:c r="AI32" t="str"/>
+      <x:c r="AJ32" t="str"/>
+      <x:c r="AK32" t="str"/>
+      <x:c r="AL32" t="str"/>
+      <x:c r="AM32" t="str"/>
+      <x:c r="AN32" t="str"/>
+      <x:c r="AO32" t="str"/>
+      <x:c r="AP32" t="str"/>
+      <x:c r="AQ32" t="str"/>
+      <x:c r="AR32" t="str"/>
+      <x:c r="AS32" t="str"/>
+      <x:c r="AT32" t="str"/>
+      <x:c r="AU32" t="str"/>
+      <x:c r="AV32" t="str"/>
+      <x:c r="AW32" t="str"/>
+      <x:c r="AX32" t="str"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>5.2</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>완료 기록 저장</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>2026-06-05</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="G33" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" t="str"/>
+      <x:c r="J33" t="str"/>
+      <x:c r="K33" t="str"/>
+      <x:c r="L33" t="str"/>
+      <x:c r="M33" t="str"/>
+      <x:c r="N33" t="str"/>
+      <x:c r="O33" t="str"/>
+      <x:c r="P33" t="str"/>
+      <x:c r="Q33" t="str"/>
+      <x:c r="R33" t="str"/>
+      <x:c r="S33" t="str"/>
+      <x:c r="T33" t="str"/>
+      <x:c r="U33" t="str"/>
+      <x:c r="V33" t="str"/>
+      <x:c r="W33" t="str"/>
+      <x:c r="X33" t="str"/>
+      <x:c r="Y33" t="str"/>
+      <x:c r="Z33" t="str"/>
+      <x:c r="AA33" t="str"/>
+      <x:c r="AB33" t="str"/>
+      <x:c r="AC33" t="str"/>
+      <x:c r="AD33" t="str"/>
+      <x:c r="AE33" t="str"/>
+      <x:c r="AF33" t="str"/>
+      <x:c r="AG33" t="str"/>
+      <x:c r="AH33" s="5" t="str"/>
+      <x:c r="AI33" s="5" t="str"/>
+      <x:c r="AJ33" s="5" t="str"/>
+      <x:c r="AK33" s="5" t="str"/>
+      <x:c r="AL33" t="str"/>
+      <x:c r="AM33" t="str"/>
+      <x:c r="AN33" t="str"/>
+      <x:c r="AO33" t="str"/>
+      <x:c r="AP33" t="str"/>
+      <x:c r="AQ33" t="str"/>
+      <x:c r="AR33" t="str"/>
+      <x:c r="AS33" t="str"/>
+      <x:c r="AT33" t="str"/>
+      <x:c r="AU33" t="str"/>
+      <x:c r="AV33" t="str"/>
+      <x:c r="AW33" t="str"/>
+      <x:c r="AX33" t="str"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>5.3</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>주간 에너지 리포트</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>2026-06-09</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>2026-06-12</x:v>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" t="str"/>
+      <x:c r="J34" t="str"/>
+      <x:c r="K34" t="str"/>
+      <x:c r="L34" t="str"/>
+      <x:c r="M34" t="str"/>
+      <x:c r="N34" t="str"/>
+      <x:c r="O34" t="str"/>
+      <x:c r="P34" t="str"/>
+      <x:c r="Q34" t="str"/>
+      <x:c r="R34" t="str"/>
+      <x:c r="S34" t="str"/>
+      <x:c r="T34" t="str"/>
+      <x:c r="U34" t="str"/>
+      <x:c r="V34" t="str"/>
+      <x:c r="W34" t="str"/>
+      <x:c r="X34" t="str"/>
+      <x:c r="Y34" t="str"/>
+      <x:c r="Z34" t="str"/>
+      <x:c r="AA34" t="str"/>
+      <x:c r="AB34" t="str"/>
+      <x:c r="AC34" t="str"/>
+      <x:c r="AD34" t="str"/>
+      <x:c r="AE34" t="str"/>
+      <x:c r="AF34" t="str"/>
+      <x:c r="AG34" t="str"/>
+      <x:c r="AH34" t="str"/>
+      <x:c r="AI34" t="str"/>
+      <x:c r="AJ34" t="str"/>
+      <x:c r="AK34" t="str"/>
+      <x:c r="AL34" s="5" t="str"/>
+      <x:c r="AM34" s="5" t="str"/>
+      <x:c r="AN34" s="5" t="str"/>
+      <x:c r="AO34" s="5" t="str"/>
+      <x:c r="AP34" t="str"/>
+      <x:c r="AQ34" t="str"/>
+      <x:c r="AR34" t="str"/>
+      <x:c r="AS34" t="str"/>
+      <x:c r="AT34" t="str"/>
+      <x:c r="AU34" t="str"/>
+      <x:c r="AV34" t="str"/>
+      <x:c r="AW34" t="str"/>
+      <x:c r="AX34" t="str"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>5.4</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>사용성 개선 및 UI 다듬기</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>2026-06-12</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="G35" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" t="str"/>
+      <x:c r="J35" t="str"/>
+      <x:c r="K35" t="str"/>
+      <x:c r="L35" t="str"/>
+      <x:c r="M35" t="str"/>
+      <x:c r="N35" t="str"/>
+      <x:c r="O35" t="str"/>
+      <x:c r="P35" t="str"/>
+      <x:c r="Q35" t="str"/>
+      <x:c r="R35" t="str"/>
+      <x:c r="S35" t="str"/>
+      <x:c r="T35" t="str"/>
+      <x:c r="U35" t="str"/>
+      <x:c r="V35" t="str"/>
+      <x:c r="W35" t="str"/>
+      <x:c r="X35" t="str"/>
+      <x:c r="Y35" t="str"/>
+      <x:c r="Z35" t="str"/>
+      <x:c r="AA35" t="str"/>
+      <x:c r="AB35" t="str"/>
+      <x:c r="AC35" t="str"/>
+      <x:c r="AD35" t="str"/>
+      <x:c r="AE35" t="str"/>
+      <x:c r="AF35" t="str"/>
+      <x:c r="AG35" t="str"/>
+      <x:c r="AH35" t="str"/>
+      <x:c r="AI35" t="str"/>
+      <x:c r="AJ35" t="str"/>
+      <x:c r="AK35" t="str"/>
+      <x:c r="AL35" t="str"/>
+      <x:c r="AM35" t="str"/>
+      <x:c r="AN35" t="str"/>
+      <x:c r="AO35" s="5" t="str"/>
+      <x:c r="AP35" s="5" t="str"/>
+      <x:c r="AQ35" s="5" t="str"/>
+      <x:c r="AR35" s="5" t="str"/>
+      <x:c r="AS35" t="str"/>
+      <x:c r="AT35" t="str"/>
+      <x:c r="AU35" t="str"/>
+      <x:c r="AV35" t="str"/>
+      <x:c r="AW35" t="str"/>
+      <x:c r="AX35" t="str"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="6" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B36" s="6" t="str">
+        <x:v>최종 테스트 및 발표</x:v>
+      </x:c>
+      <x:c r="C36" s="6" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D36" s="6" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E36" s="6" t="str">
+        <x:v>2026-06-16</x:v>
+      </x:c>
+      <x:c r="F36" s="6" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="G36" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H36" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" s="6" t="str"/>
+      <x:c r="J36" s="6" t="str"/>
+      <x:c r="K36" s="6" t="str"/>
+      <x:c r="L36" s="6" t="str"/>
+      <x:c r="M36" s="6" t="str"/>
+      <x:c r="N36" s="6" t="str"/>
+      <x:c r="O36" s="6" t="str"/>
+      <x:c r="P36" s="6" t="str"/>
+      <x:c r="Q36" s="6" t="str"/>
+      <x:c r="R36" s="6" t="str"/>
+      <x:c r="S36" s="6" t="str"/>
+      <x:c r="T36" s="6" t="str"/>
+      <x:c r="U36" s="6" t="str"/>
+      <x:c r="V36" s="6" t="str"/>
+      <x:c r="W36" s="6" t="str"/>
+      <x:c r="X36" s="6" t="str"/>
+      <x:c r="Y36" s="6" t="str"/>
+      <x:c r="Z36" s="6" t="str"/>
+      <x:c r="AA36" s="6" t="str"/>
+      <x:c r="AB36" s="6" t="str"/>
+      <x:c r="AC36" s="6" t="str"/>
+      <x:c r="AD36" s="6" t="str"/>
+      <x:c r="AE36" s="6" t="str"/>
+      <x:c r="AF36" s="6" t="str"/>
+      <x:c r="AG36" s="6" t="str"/>
+      <x:c r="AH36" s="6" t="str"/>
+      <x:c r="AI36" s="6" t="str"/>
+      <x:c r="AJ36" s="6" t="str"/>
+      <x:c r="AK36" s="6" t="str"/>
+      <x:c r="AL36" s="6" t="str"/>
+      <x:c r="AM36" s="6" t="str"/>
+      <x:c r="AN36" s="6" t="str"/>
+      <x:c r="AO36" s="6" t="str"/>
+      <x:c r="AP36" s="6" t="str"/>
+      <x:c r="AQ36" s="6" t="str"/>
+      <x:c r="AR36" s="6" t="str"/>
+      <x:c r="AS36" s="6" t="str"/>
+      <x:c r="AT36" s="6" t="str"/>
+      <x:c r="AU36" s="6" t="str"/>
+      <x:c r="AV36" s="6" t="str"/>
+      <x:c r="AW36" s="6" t="str"/>
+      <x:c r="AX36" s="6" t="str"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>6.1</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>사용자 시나리오 테스트</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>2026-06-16</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>2026-06-18</x:v>
+      </x:c>
+      <x:c r="G37" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I37" t="str"/>
+      <x:c r="J37" t="str"/>
+      <x:c r="K37" t="str"/>
+      <x:c r="L37" t="str"/>
+      <x:c r="M37" t="str"/>
+      <x:c r="N37" t="str"/>
+      <x:c r="O37" t="str"/>
+      <x:c r="P37" t="str"/>
+      <x:c r="Q37" t="str"/>
+      <x:c r="R37" t="str"/>
+      <x:c r="S37" t="str"/>
+      <x:c r="T37" t="str"/>
+      <x:c r="U37" t="str"/>
+      <x:c r="V37" t="str"/>
+      <x:c r="W37" t="str"/>
+      <x:c r="X37" t="str"/>
+      <x:c r="Y37" t="str"/>
+      <x:c r="Z37" t="str"/>
+      <x:c r="AA37" t="str"/>
+      <x:c r="AB37" t="str"/>
+      <x:c r="AC37" t="str"/>
+      <x:c r="AD37" t="str"/>
+      <x:c r="AE37" t="str"/>
+      <x:c r="AF37" t="str"/>
+      <x:c r="AG37" t="str"/>
+      <x:c r="AH37" t="str"/>
+      <x:c r="AI37" t="str"/>
+      <x:c r="AJ37" t="str"/>
+      <x:c r="AK37" t="str"/>
+      <x:c r="AL37" t="str"/>
+      <x:c r="AM37" t="str"/>
+      <x:c r="AN37" t="str"/>
+      <x:c r="AO37" t="str"/>
+      <x:c r="AP37" t="str"/>
+      <x:c r="AQ37" t="str"/>
+      <x:c r="AR37" t="str"/>
+      <x:c r="AS37" s="5" t="str"/>
+      <x:c r="AT37" s="5" t="str"/>
+      <x:c r="AU37" s="5" t="str"/>
+      <x:c r="AV37" t="str"/>
+      <x:c r="AW37" t="str"/>
+      <x:c r="AX37" t="str"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>6.2</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>README와 실행 방법 최종 정리</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>2026-06-18</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="G38" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I38" t="str"/>
+      <x:c r="J38" t="str"/>
+      <x:c r="K38" t="str"/>
+      <x:c r="L38" t="str"/>
+      <x:c r="M38" t="str"/>
+      <x:c r="N38" t="str"/>
+      <x:c r="O38" t="str"/>
+      <x:c r="P38" t="str"/>
+      <x:c r="Q38" t="str"/>
+      <x:c r="R38" t="str"/>
+      <x:c r="S38" t="str"/>
+      <x:c r="T38" t="str"/>
+      <x:c r="U38" t="str"/>
+      <x:c r="V38" t="str"/>
+      <x:c r="W38" t="str"/>
+      <x:c r="X38" t="str"/>
+      <x:c r="Y38" t="str"/>
+      <x:c r="Z38" t="str"/>
+      <x:c r="AA38" t="str"/>
+      <x:c r="AB38" t="str"/>
+      <x:c r="AC38" t="str"/>
+      <x:c r="AD38" t="str"/>
+      <x:c r="AE38" t="str"/>
+      <x:c r="AF38" t="str"/>
+      <x:c r="AG38" t="str"/>
+      <x:c r="AH38" t="str"/>
+      <x:c r="AI38" t="str"/>
+      <x:c r="AJ38" t="str"/>
+      <x:c r="AK38" t="str"/>
+      <x:c r="AL38" t="str"/>
+      <x:c r="AM38" t="str"/>
+      <x:c r="AN38" t="str"/>
+      <x:c r="AO38" t="str"/>
+      <x:c r="AP38" t="str"/>
+      <x:c r="AQ38" t="str"/>
+      <x:c r="AR38" t="str"/>
+      <x:c r="AS38" t="str"/>
+      <x:c r="AT38" t="str"/>
+      <x:c r="AU38" s="5" t="str"/>
+      <x:c r="AV38" s="5" t="str"/>
+      <x:c r="AW38" t="str"/>
+      <x:c r="AX38" t="str"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>6.3</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>발표 리허설 및 PDF 최종 점검</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>2026-06-19</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
+      <x:c r="G39" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I39" t="str"/>
+      <x:c r="J39" t="str"/>
+      <x:c r="K39" t="str"/>
+      <x:c r="L39" t="str"/>
+      <x:c r="M39" t="str"/>
+      <x:c r="N39" t="str"/>
+      <x:c r="O39" t="str"/>
+      <x:c r="P39" t="str"/>
+      <x:c r="Q39" t="str"/>
+      <x:c r="R39" t="str"/>
+      <x:c r="S39" t="str"/>
+      <x:c r="T39" t="str"/>
+      <x:c r="U39" t="str"/>
+      <x:c r="V39" t="str"/>
+      <x:c r="W39" t="str"/>
+      <x:c r="X39" t="str"/>
+      <x:c r="Y39" t="str"/>
+      <x:c r="Z39" t="str"/>
+      <x:c r="AA39" t="str"/>
+      <x:c r="AB39" t="str"/>
+      <x:c r="AC39" t="str"/>
+      <x:c r="AD39" t="str"/>
+      <x:c r="AE39" t="str"/>
+      <x:c r="AF39" t="str"/>
+      <x:c r="AG39" t="str"/>
+      <x:c r="AH39" t="str"/>
+      <x:c r="AI39" t="str"/>
+      <x:c r="AJ39" t="str"/>
+      <x:c r="AK39" t="str"/>
+      <x:c r="AL39" t="str"/>
+      <x:c r="AM39" t="str"/>
+      <x:c r="AN39" t="str"/>
+      <x:c r="AO39" t="str"/>
+      <x:c r="AP39" t="str"/>
+      <x:c r="AQ39" t="str"/>
+      <x:c r="AR39" t="str"/>
+      <x:c r="AS39" t="str"/>
+      <x:c r="AT39" t="str"/>
+      <x:c r="AU39" t="str"/>
+      <x:c r="AV39" s="5" t="str"/>
+      <x:c r="AW39" s="5" t="str"/>
+      <x:c r="AX39" s="5" t="str"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="11" t="str">
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>최종 발표</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>Milestone</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="G40" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="str"/>
+      <x:c r="J40" s="11" t="str"/>
+      <x:c r="K40" s="11" t="str"/>
+      <x:c r="L40" s="11" t="str"/>
+      <x:c r="M40" s="11" t="str"/>
+      <x:c r="N40" s="11" t="str"/>
+      <x:c r="O40" s="11" t="str"/>
+      <x:c r="P40" s="11" t="str"/>
+      <x:c r="Q40" s="11" t="str"/>
+      <x:c r="R40" s="11" t="str"/>
+      <x:c r="S40" s="11" t="str"/>
+      <x:c r="T40" s="11" t="str"/>
+      <x:c r="U40" s="11" t="str"/>
+      <x:c r="V40" s="11" t="str"/>
+      <x:c r="W40" s="11" t="str"/>
+      <x:c r="X40" s="11" t="str"/>
+      <x:c r="Y40" s="11" t="str"/>
+      <x:c r="Z40" s="11" t="str"/>
+      <x:c r="AA40" s="11" t="str"/>
+      <x:c r="AB40" s="11" t="str"/>
+      <x:c r="AC40" s="11" t="str"/>
+      <x:c r="AD40" s="11" t="str"/>
+      <x:c r="AE40" s="11" t="str"/>
+      <x:c r="AF40" s="11" t="str"/>
+      <x:c r="AG40" s="11" t="str"/>
+      <x:c r="AH40" s="11" t="str"/>
+      <x:c r="AI40" s="11" t="str"/>
+      <x:c r="AJ40" s="11" t="str"/>
+      <x:c r="AK40" s="11" t="str"/>
+      <x:c r="AL40" s="11" t="str"/>
+      <x:c r="AM40" s="11" t="str"/>
+      <x:c r="AN40" s="11" t="str"/>
+      <x:c r="AO40" s="11" t="str"/>
+      <x:c r="AP40" s="11" t="str"/>
+      <x:c r="AQ40" s="11" t="str"/>
+      <x:c r="AR40" s="11" t="str"/>
+      <x:c r="AS40" s="11" t="str"/>
+      <x:c r="AT40" s="11" t="str"/>
+      <x:c r="AU40" s="11" t="str"/>
+      <x:c r="AV40" s="11" t="str"/>
+      <x:c r="AW40" s="11" t="str"/>
+      <x:c r="AX40" s="11" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2389,16 +3150,16 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="13" t="str">
+      <x:c r="A1" s="16" t="str">
         <x:v>구분</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="16" t="str">
         <x:v>설명</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C1" s="16" t="str">
         <x:v>프로젝트 적용</x:v>
       </x:c>
-      <x:c r="D1" s="13" t="str">
+      <x:c r="D1" s="16" t="str">
         <x:v>발표 포인트</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Polish PDF WBS layout and formal WBS
</commit_message>
<xml_diff>
--- a/Energy_Budget_WBS_Gantt.xlsx
+++ b/Energy_Budget_WBS_Gantt.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS Gantt" sheetId="1" r:id="R085271602f764c96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rbf8e628ebabd4a70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS Gantt" sheetId="1" r:id="Redbfed52b98346ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R7f7f221ea9394c60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -327,7 +327,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Energy Budget WBS &amp; Gantt Chart</x:v>
+        <x:v>Energy Budget Formal WBS &amp; Gantt Chart</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str"/>
       <x:c r="C1" s="2" t="str"/>
@@ -483,10 +483,10 @@
         <x:v>Finish Date</x:v>
       </x:c>
       <x:c r="G3" s="4" t="str">
-        <x:v>W</x:v>
+        <x:v>Duration</x:v>
       </x:c>
       <x:c r="H3" s="4" t="str">
-        <x:v>%</x:v>
+        <x:v>Progress</x:v>
       </x:c>
       <x:c r="I3" s="4" t="str">
         <x:v>1</x:v>
@@ -2060,13 +2060,13 @@
         <x:v>2026-05-27</x:v>
       </x:c>
       <x:c r="F25" s="6" t="str">
-        <x:v>2026-05-31</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="G25" s="6" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H25" s="6" t="n">
-        <x:v>85</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I25" s="6" t="str"/>
       <x:c r="J25" s="6" t="str"/>
@@ -2089,8 +2089,8 @@
       <x:c r="AA25" s="13" t="str"/>
       <x:c r="AB25" s="13" t="str"/>
       <x:c r="AC25" s="13" t="str"/>
-      <x:c r="AD25" s="6" t="str"/>
-      <x:c r="AE25" s="6" t="str"/>
+      <x:c r="AD25" s="13" t="str"/>
+      <x:c r="AE25" s="13" t="str"/>
       <x:c r="AF25" s="6" t="str"/>
       <x:c r="AG25" s="6" t="str"/>
       <x:c r="AH25" s="6" t="str"/>
@@ -2264,10 +2264,10 @@
         <x:v>2026-05-28</x:v>
       </x:c>
       <x:c r="F28" t="str">
-        <x:v>2026-05-28</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="G28" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H28" t="n">
         <x:v>100</x:v>
@@ -2290,11 +2290,11 @@
       <x:c r="X28" t="str"/>
       <x:c r="Y28" t="str"/>
       <x:c r="Z28" s="9" t="str"/>
-      <x:c r="AA28" t="str"/>
-      <x:c r="AB28" t="str"/>
-      <x:c r="AC28" t="str"/>
-      <x:c r="AD28" t="str"/>
-      <x:c r="AE28" t="str"/>
+      <x:c r="AA28" s="9" t="str"/>
+      <x:c r="AB28" s="9" t="str"/>
+      <x:c r="AC28" s="9" t="str"/>
+      <x:c r="AD28" s="9" t="str"/>
+      <x:c r="AE28" s="9" t="str"/>
       <x:c r="AF28" t="str"/>
       <x:c r="AG28" t="str"/>
       <x:c r="AH28" t="str"/>
@@ -2320,25 +2320,25 @@
         <x:v>4.4</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>WBS Gantt 엑셀 최신화</x:v>
+        <x:v>WBS 진행 상태 발표자료 반영</x:v>
       </x:c>
       <x:c r="C29" t="str">
         <x:v>정원식</x:v>
       </x:c>
-      <x:c r="D29" s="14" t="str">
-        <x:v>In Progress</x:v>
+      <x:c r="D29" s="8" t="str">
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E29" t="str">
-        <x:v>2026-05-28</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="F29" t="str">
-        <x:v>2026-05-29</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="G29" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H29" t="n">
-        <x:v>70</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I29" t="str"/>
       <x:c r="J29" t="str"/>
@@ -2357,12 +2357,12 @@
       <x:c r="W29" t="str"/>
       <x:c r="X29" t="str"/>
       <x:c r="Y29" t="str"/>
-      <x:c r="Z29" s="15" t="str"/>
-      <x:c r="AA29" s="15" t="str"/>
+      <x:c r="Z29" t="str"/>
+      <x:c r="AA29" t="str"/>
       <x:c r="AB29" t="str"/>
       <x:c r="AC29" t="str"/>
       <x:c r="AD29" t="str"/>
-      <x:c r="AE29" t="str"/>
+      <x:c r="AE29" s="9" t="str"/>
       <x:c r="AF29" t="str"/>
       <x:c r="AG29" t="str"/>
       <x:c r="AH29" t="str"/>
@@ -2388,7 +2388,7 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>GitHub Pages 배포 점검</x:v>
+        <x:v>WBS Gantt 엑셀 FM 정리</x:v>
       </x:c>
       <x:c r="C30" t="str">
         <x:v>정원식</x:v>
@@ -2397,16 +2397,16 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E30" t="str">
-        <x:v>2026-05-29</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="F30" t="str">
-        <x:v>2026-05-31</x:v>
+        <x:v>2026-06-02</x:v>
       </x:c>
       <x:c r="G30" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H30" t="n">
-        <x:v>60</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="I30" t="str"/>
       <x:c r="J30" t="str"/>
@@ -2426,11 +2426,11 @@
       <x:c r="X30" t="str"/>
       <x:c r="Y30" t="str"/>
       <x:c r="Z30" t="str"/>
-      <x:c r="AA30" s="15" t="str"/>
-      <x:c r="AB30" s="15" t="str"/>
-      <x:c r="AC30" s="15" t="str"/>
+      <x:c r="AA30" t="str"/>
+      <x:c r="AB30" t="str"/>
+      <x:c r="AC30" t="str"/>
       <x:c r="AD30" t="str"/>
-      <x:c r="AE30" t="str"/>
+      <x:c r="AE30" s="15" t="str"/>
       <x:c r="AF30" t="str"/>
       <x:c r="AG30" t="str"/>
       <x:c r="AH30" t="str"/>
@@ -2452,147 +2452,147 @@
       <x:c r="AX30" t="str"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="6" t="str">
+      <x:c r="A31" t="str">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>GitHub Pages 배포 점검</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D31" s="14" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H31" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I31" t="str"/>
+      <x:c r="J31" t="str"/>
+      <x:c r="K31" t="str"/>
+      <x:c r="L31" t="str"/>
+      <x:c r="M31" t="str"/>
+      <x:c r="N31" t="str"/>
+      <x:c r="O31" t="str"/>
+      <x:c r="P31" t="str"/>
+      <x:c r="Q31" t="str"/>
+      <x:c r="R31" t="str"/>
+      <x:c r="S31" t="str"/>
+      <x:c r="T31" t="str"/>
+      <x:c r="U31" t="str"/>
+      <x:c r="V31" t="str"/>
+      <x:c r="W31" t="str"/>
+      <x:c r="X31" t="str"/>
+      <x:c r="Y31" t="str"/>
+      <x:c r="Z31" t="str"/>
+      <x:c r="AA31" t="str"/>
+      <x:c r="AB31" t="str"/>
+      <x:c r="AC31" t="str"/>
+      <x:c r="AD31" t="str"/>
+      <x:c r="AE31" s="15" t="str"/>
+      <x:c r="AF31" t="str"/>
+      <x:c r="AG31" t="str"/>
+      <x:c r="AH31" t="str"/>
+      <x:c r="AI31" t="str"/>
+      <x:c r="AJ31" t="str"/>
+      <x:c r="AK31" t="str"/>
+      <x:c r="AL31" t="str"/>
+      <x:c r="AM31" t="str"/>
+      <x:c r="AN31" t="str"/>
+      <x:c r="AO31" t="str"/>
+      <x:c r="AP31" t="str"/>
+      <x:c r="AQ31" t="str"/>
+      <x:c r="AR31" t="str"/>
+      <x:c r="AS31" t="str"/>
+      <x:c r="AT31" t="str"/>
+      <x:c r="AU31" t="str"/>
+      <x:c r="AV31" t="str"/>
+      <x:c r="AW31" t="str"/>
+      <x:c r="AX31" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="6" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B31" s="6" t="str">
+      <x:c r="B32" s="6" t="str">
         <x:v>추가 기능 개발</x:v>
       </x:c>
-      <x:c r="C31" s="6" t="str">
+      <x:c r="C32" s="6" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="D31" s="6" t="str">
+      <x:c r="D32" s="6" t="str">
         <x:v>Not Started</x:v>
       </x:c>
-      <x:c r="E31" s="6" t="str">
+      <x:c r="E32" s="6" t="str">
         <x:v>2026-06-02</x:v>
       </x:c>
-      <x:c r="F31" s="6" t="str">
+      <x:c r="F32" s="6" t="str">
         <x:v>2026-06-15</x:v>
       </x:c>
-      <x:c r="G31" s="6" t="n">
+      <x:c r="G32" s="6" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="H31" s="6" t="n">
+      <x:c r="H32" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I31" s="6" t="str"/>
-      <x:c r="J31" s="6" t="str"/>
-      <x:c r="K31" s="6" t="str"/>
-      <x:c r="L31" s="6" t="str"/>
-      <x:c r="M31" s="6" t="str"/>
-      <x:c r="N31" s="6" t="str"/>
-      <x:c r="O31" s="6" t="str"/>
-      <x:c r="P31" s="6" t="str"/>
-      <x:c r="Q31" s="6" t="str"/>
-      <x:c r="R31" s="6" t="str"/>
-      <x:c r="S31" s="6" t="str"/>
-      <x:c r="T31" s="6" t="str"/>
-      <x:c r="U31" s="6" t="str"/>
-      <x:c r="V31" s="6" t="str"/>
-      <x:c r="W31" s="6" t="str"/>
-      <x:c r="X31" s="6" t="str"/>
-      <x:c r="Y31" s="6" t="str"/>
-      <x:c r="Z31" s="6" t="str"/>
-      <x:c r="AA31" s="6" t="str"/>
-      <x:c r="AB31" s="6" t="str"/>
-      <x:c r="AC31" s="6" t="str"/>
-      <x:c r="AD31" s="6" t="str"/>
-      <x:c r="AE31" s="6" t="str"/>
-      <x:c r="AF31" s="6" t="str"/>
-      <x:c r="AG31" s="6" t="str"/>
-      <x:c r="AH31" s="6" t="str"/>
-      <x:c r="AI31" s="6" t="str"/>
-      <x:c r="AJ31" s="6" t="str"/>
-      <x:c r="AK31" s="6" t="str"/>
-      <x:c r="AL31" s="6" t="str"/>
-      <x:c r="AM31" s="6" t="str"/>
-      <x:c r="AN31" s="6" t="str"/>
-      <x:c r="AO31" s="6" t="str"/>
-      <x:c r="AP31" s="6" t="str"/>
-      <x:c r="AQ31" s="6" t="str"/>
-      <x:c r="AR31" s="6" t="str"/>
-      <x:c r="AS31" s="6" t="str"/>
-      <x:c r="AT31" s="6" t="str"/>
-      <x:c r="AU31" s="6" t="str"/>
-      <x:c r="AV31" s="6" t="str"/>
-      <x:c r="AW31" s="6" t="str"/>
-      <x:c r="AX31" s="6" t="str"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" t="str">
-        <x:v>5.1</x:v>
-      </x:c>
-      <x:c r="B32" t="str">
-        <x:v>일일 계획 저장 기능</x:v>
-      </x:c>
-      <x:c r="C32" t="str">
-        <x:v>정원식</x:v>
-      </x:c>
-      <x:c r="D32" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E32" t="str">
-        <x:v>2026-06-02</x:v>
-      </x:c>
-      <x:c r="F32" t="str">
-        <x:v>2026-06-05</x:v>
-      </x:c>
-      <x:c r="G32" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I32" t="str"/>
-      <x:c r="J32" t="str"/>
-      <x:c r="K32" t="str"/>
-      <x:c r="L32" t="str"/>
-      <x:c r="M32" t="str"/>
-      <x:c r="N32" t="str"/>
-      <x:c r="O32" t="str"/>
-      <x:c r="P32" t="str"/>
-      <x:c r="Q32" t="str"/>
-      <x:c r="R32" t="str"/>
-      <x:c r="S32" t="str"/>
-      <x:c r="T32" t="str"/>
-      <x:c r="U32" t="str"/>
-      <x:c r="V32" t="str"/>
-      <x:c r="W32" t="str"/>
-      <x:c r="X32" t="str"/>
-      <x:c r="Y32" t="str"/>
-      <x:c r="Z32" t="str"/>
-      <x:c r="AA32" t="str"/>
-      <x:c r="AB32" t="str"/>
-      <x:c r="AC32" t="str"/>
-      <x:c r="AD32" t="str"/>
-      <x:c r="AE32" s="5" t="str"/>
-      <x:c r="AF32" s="5" t="str"/>
-      <x:c r="AG32" s="5" t="str"/>
-      <x:c r="AH32" s="5" t="str"/>
-      <x:c r="AI32" t="str"/>
-      <x:c r="AJ32" t="str"/>
-      <x:c r="AK32" t="str"/>
-      <x:c r="AL32" t="str"/>
-      <x:c r="AM32" t="str"/>
-      <x:c r="AN32" t="str"/>
-      <x:c r="AO32" t="str"/>
-      <x:c r="AP32" t="str"/>
-      <x:c r="AQ32" t="str"/>
-      <x:c r="AR32" t="str"/>
-      <x:c r="AS32" t="str"/>
-      <x:c r="AT32" t="str"/>
-      <x:c r="AU32" t="str"/>
-      <x:c r="AV32" t="str"/>
-      <x:c r="AW32" t="str"/>
-      <x:c r="AX32" t="str"/>
+      <x:c r="I32" s="6" t="str"/>
+      <x:c r="J32" s="6" t="str"/>
+      <x:c r="K32" s="6" t="str"/>
+      <x:c r="L32" s="6" t="str"/>
+      <x:c r="M32" s="6" t="str"/>
+      <x:c r="N32" s="6" t="str"/>
+      <x:c r="O32" s="6" t="str"/>
+      <x:c r="P32" s="6" t="str"/>
+      <x:c r="Q32" s="6" t="str"/>
+      <x:c r="R32" s="6" t="str"/>
+      <x:c r="S32" s="6" t="str"/>
+      <x:c r="T32" s="6" t="str"/>
+      <x:c r="U32" s="6" t="str"/>
+      <x:c r="V32" s="6" t="str"/>
+      <x:c r="W32" s="6" t="str"/>
+      <x:c r="X32" s="6" t="str"/>
+      <x:c r="Y32" s="6" t="str"/>
+      <x:c r="Z32" s="6" t="str"/>
+      <x:c r="AA32" s="6" t="str"/>
+      <x:c r="AB32" s="6" t="str"/>
+      <x:c r="AC32" s="6" t="str"/>
+      <x:c r="AD32" s="6" t="str"/>
+      <x:c r="AE32" s="6" t="str"/>
+      <x:c r="AF32" s="6" t="str"/>
+      <x:c r="AG32" s="6" t="str"/>
+      <x:c r="AH32" s="6" t="str"/>
+      <x:c r="AI32" s="6" t="str"/>
+      <x:c r="AJ32" s="6" t="str"/>
+      <x:c r="AK32" s="6" t="str"/>
+      <x:c r="AL32" s="6" t="str"/>
+      <x:c r="AM32" s="6" t="str"/>
+      <x:c r="AN32" s="6" t="str"/>
+      <x:c r="AO32" s="6" t="str"/>
+      <x:c r="AP32" s="6" t="str"/>
+      <x:c r="AQ32" s="6" t="str"/>
+      <x:c r="AR32" s="6" t="str"/>
+      <x:c r="AS32" s="6" t="str"/>
+      <x:c r="AT32" s="6" t="str"/>
+      <x:c r="AU32" s="6" t="str"/>
+      <x:c r="AV32" s="6" t="str"/>
+      <x:c r="AW32" s="6" t="str"/>
+      <x:c r="AX32" s="6" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>5.2</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>완료 기록 저장</x:v>
+        <x:v>일일 계획 저장 기능</x:v>
       </x:c>
       <x:c r="C33" t="str">
         <x:v>정원식</x:v>
@@ -2601,10 +2601,10 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E33" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
         <x:v>2026-06-05</x:v>
-      </x:c>
-      <x:c r="F33" t="str">
-        <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="G33" t="n">
         <x:v>4</x:v>
@@ -2634,13 +2634,13 @@
       <x:c r="AB33" t="str"/>
       <x:c r="AC33" t="str"/>
       <x:c r="AD33" t="str"/>
-      <x:c r="AE33" t="str"/>
-      <x:c r="AF33" t="str"/>
-      <x:c r="AG33" t="str"/>
+      <x:c r="AE33" s="5" t="str"/>
+      <x:c r="AF33" s="5" t="str"/>
+      <x:c r="AG33" s="5" t="str"/>
       <x:c r="AH33" s="5" t="str"/>
-      <x:c r="AI33" s="5" t="str"/>
-      <x:c r="AJ33" s="5" t="str"/>
-      <x:c r="AK33" s="5" t="str"/>
+      <x:c r="AI33" t="str"/>
+      <x:c r="AJ33" t="str"/>
+      <x:c r="AK33" t="str"/>
       <x:c r="AL33" t="str"/>
       <x:c r="AM33" t="str"/>
       <x:c r="AN33" t="str"/>
@@ -2657,10 +2657,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>5.3</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>주간 에너지 리포트</x:v>
+        <x:v>완료 기록 저장</x:v>
       </x:c>
       <x:c r="C34" t="str">
         <x:v>정원식</x:v>
@@ -2669,10 +2669,10 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E34" t="str">
-        <x:v>2026-06-09</x:v>
+        <x:v>2026-06-05</x:v>
       </x:c>
       <x:c r="F34" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="G34" t="n">
         <x:v>4</x:v>
@@ -2705,14 +2705,14 @@
       <x:c r="AE34" t="str"/>
       <x:c r="AF34" t="str"/>
       <x:c r="AG34" t="str"/>
-      <x:c r="AH34" t="str"/>
-      <x:c r="AI34" t="str"/>
-      <x:c r="AJ34" t="str"/>
-      <x:c r="AK34" t="str"/>
-      <x:c r="AL34" s="5" t="str"/>
-      <x:c r="AM34" s="5" t="str"/>
-      <x:c r="AN34" s="5" t="str"/>
-      <x:c r="AO34" s="5" t="str"/>
+      <x:c r="AH34" s="5" t="str"/>
+      <x:c r="AI34" s="5" t="str"/>
+      <x:c r="AJ34" s="5" t="str"/>
+      <x:c r="AK34" s="5" t="str"/>
+      <x:c r="AL34" t="str"/>
+      <x:c r="AM34" t="str"/>
+      <x:c r="AN34" t="str"/>
+      <x:c r="AO34" t="str"/>
       <x:c r="AP34" t="str"/>
       <x:c r="AQ34" t="str"/>
       <x:c r="AR34" t="str"/>
@@ -2725,10 +2725,10 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>5.4</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>사용성 개선 및 UI 다듬기</x:v>
+        <x:v>주간 에너지 리포트</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>정원식</x:v>
@@ -2737,10 +2737,10 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E35" t="str">
+        <x:v>2026-06-09</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
         <x:v>2026-06-12</x:v>
-      </x:c>
-      <x:c r="F35" t="str">
-        <x:v>2026-06-15</x:v>
       </x:c>
       <x:c r="G35" t="n">
         <x:v>4</x:v>
@@ -2777,13 +2777,13 @@
       <x:c r="AI35" t="str"/>
       <x:c r="AJ35" t="str"/>
       <x:c r="AK35" t="str"/>
-      <x:c r="AL35" t="str"/>
-      <x:c r="AM35" t="str"/>
-      <x:c r="AN35" t="str"/>
+      <x:c r="AL35" s="5" t="str"/>
+      <x:c r="AM35" s="5" t="str"/>
+      <x:c r="AN35" s="5" t="str"/>
       <x:c r="AO35" s="5" t="str"/>
-      <x:c r="AP35" s="5" t="str"/>
-      <x:c r="AQ35" s="5" t="str"/>
-      <x:c r="AR35" s="5" t="str"/>
+      <x:c r="AP35" t="str"/>
+      <x:c r="AQ35" t="str"/>
+      <x:c r="AR35" t="str"/>
       <x:c r="AS35" t="str"/>
       <x:c r="AT35" t="str"/>
       <x:c r="AU35" t="str"/>
@@ -2792,147 +2792,147 @@
       <x:c r="AX35" t="str"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="6" t="str">
+      <x:c r="A36" t="str">
+        <x:v>5.4</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>사용성 개선 및 UI 다듬기</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>2026-06-12</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>2026-06-15</x:v>
+      </x:c>
+      <x:c r="G36" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I36" t="str"/>
+      <x:c r="J36" t="str"/>
+      <x:c r="K36" t="str"/>
+      <x:c r="L36" t="str"/>
+      <x:c r="M36" t="str"/>
+      <x:c r="N36" t="str"/>
+      <x:c r="O36" t="str"/>
+      <x:c r="P36" t="str"/>
+      <x:c r="Q36" t="str"/>
+      <x:c r="R36" t="str"/>
+      <x:c r="S36" t="str"/>
+      <x:c r="T36" t="str"/>
+      <x:c r="U36" t="str"/>
+      <x:c r="V36" t="str"/>
+      <x:c r="W36" t="str"/>
+      <x:c r="X36" t="str"/>
+      <x:c r="Y36" t="str"/>
+      <x:c r="Z36" t="str"/>
+      <x:c r="AA36" t="str"/>
+      <x:c r="AB36" t="str"/>
+      <x:c r="AC36" t="str"/>
+      <x:c r="AD36" t="str"/>
+      <x:c r="AE36" t="str"/>
+      <x:c r="AF36" t="str"/>
+      <x:c r="AG36" t="str"/>
+      <x:c r="AH36" t="str"/>
+      <x:c r="AI36" t="str"/>
+      <x:c r="AJ36" t="str"/>
+      <x:c r="AK36" t="str"/>
+      <x:c r="AL36" t="str"/>
+      <x:c r="AM36" t="str"/>
+      <x:c r="AN36" t="str"/>
+      <x:c r="AO36" s="5" t="str"/>
+      <x:c r="AP36" s="5" t="str"/>
+      <x:c r="AQ36" s="5" t="str"/>
+      <x:c r="AR36" s="5" t="str"/>
+      <x:c r="AS36" t="str"/>
+      <x:c r="AT36" t="str"/>
+      <x:c r="AU36" t="str"/>
+      <x:c r="AV36" t="str"/>
+      <x:c r="AW36" t="str"/>
+      <x:c r="AX36" t="str"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="6" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B36" s="6" t="str">
+      <x:c r="B37" s="6" t="str">
         <x:v>최종 테스트 및 발표</x:v>
       </x:c>
-      <x:c r="C36" s="6" t="str">
+      <x:c r="C37" s="6" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="D36" s="6" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E36" s="6" t="str">
+      <x:c r="D37" s="6" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="E37" s="6" t="str">
         <x:v>2026-06-16</x:v>
       </x:c>
-      <x:c r="F36" s="6" t="str">
+      <x:c r="F37" s="6" t="str">
         <x:v>2026-06-22</x:v>
       </x:c>
-      <x:c r="G36" s="6" t="n">
+      <x:c r="G37" s="6" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="H36" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I36" s="6" t="str"/>
-      <x:c r="J36" s="6" t="str"/>
-      <x:c r="K36" s="6" t="str"/>
-      <x:c r="L36" s="6" t="str"/>
-      <x:c r="M36" s="6" t="str"/>
-      <x:c r="N36" s="6" t="str"/>
-      <x:c r="O36" s="6" t="str"/>
-      <x:c r="P36" s="6" t="str"/>
-      <x:c r="Q36" s="6" t="str"/>
-      <x:c r="R36" s="6" t="str"/>
-      <x:c r="S36" s="6" t="str"/>
-      <x:c r="T36" s="6" t="str"/>
-      <x:c r="U36" s="6" t="str"/>
-      <x:c r="V36" s="6" t="str"/>
-      <x:c r="W36" s="6" t="str"/>
-      <x:c r="X36" s="6" t="str"/>
-      <x:c r="Y36" s="6" t="str"/>
-      <x:c r="Z36" s="6" t="str"/>
-      <x:c r="AA36" s="6" t="str"/>
-      <x:c r="AB36" s="6" t="str"/>
-      <x:c r="AC36" s="6" t="str"/>
-      <x:c r="AD36" s="6" t="str"/>
-      <x:c r="AE36" s="6" t="str"/>
-      <x:c r="AF36" s="6" t="str"/>
-      <x:c r="AG36" s="6" t="str"/>
-      <x:c r="AH36" s="6" t="str"/>
-      <x:c r="AI36" s="6" t="str"/>
-      <x:c r="AJ36" s="6" t="str"/>
-      <x:c r="AK36" s="6" t="str"/>
-      <x:c r="AL36" s="6" t="str"/>
-      <x:c r="AM36" s="6" t="str"/>
-      <x:c r="AN36" s="6" t="str"/>
-      <x:c r="AO36" s="6" t="str"/>
-      <x:c r="AP36" s="6" t="str"/>
-      <x:c r="AQ36" s="6" t="str"/>
-      <x:c r="AR36" s="6" t="str"/>
-      <x:c r="AS36" s="6" t="str"/>
-      <x:c r="AT36" s="6" t="str"/>
-      <x:c r="AU36" s="6" t="str"/>
-      <x:c r="AV36" s="6" t="str"/>
-      <x:c r="AW36" s="6" t="str"/>
-      <x:c r="AX36" s="6" t="str"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
-        <x:v>6.1</x:v>
-      </x:c>
-      <x:c r="B37" t="str">
-        <x:v>사용자 시나리오 테스트</x:v>
-      </x:c>
-      <x:c r="C37" t="str">
-        <x:v>정원식</x:v>
-      </x:c>
-      <x:c r="D37" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="E37" t="str">
-        <x:v>2026-06-16</x:v>
-      </x:c>
-      <x:c r="F37" t="str">
-        <x:v>2026-06-18</x:v>
-      </x:c>
-      <x:c r="G37" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H37" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I37" t="str"/>
-      <x:c r="J37" t="str"/>
-      <x:c r="K37" t="str"/>
-      <x:c r="L37" t="str"/>
-      <x:c r="M37" t="str"/>
-      <x:c r="N37" t="str"/>
-      <x:c r="O37" t="str"/>
-      <x:c r="P37" t="str"/>
-      <x:c r="Q37" t="str"/>
-      <x:c r="R37" t="str"/>
-      <x:c r="S37" t="str"/>
-      <x:c r="T37" t="str"/>
-      <x:c r="U37" t="str"/>
-      <x:c r="V37" t="str"/>
-      <x:c r="W37" t="str"/>
-      <x:c r="X37" t="str"/>
-      <x:c r="Y37" t="str"/>
-      <x:c r="Z37" t="str"/>
-      <x:c r="AA37" t="str"/>
-      <x:c r="AB37" t="str"/>
-      <x:c r="AC37" t="str"/>
-      <x:c r="AD37" t="str"/>
-      <x:c r="AE37" t="str"/>
-      <x:c r="AF37" t="str"/>
-      <x:c r="AG37" t="str"/>
-      <x:c r="AH37" t="str"/>
-      <x:c r="AI37" t="str"/>
-      <x:c r="AJ37" t="str"/>
-      <x:c r="AK37" t="str"/>
-      <x:c r="AL37" t="str"/>
-      <x:c r="AM37" t="str"/>
-      <x:c r="AN37" t="str"/>
-      <x:c r="AO37" t="str"/>
-      <x:c r="AP37" t="str"/>
-      <x:c r="AQ37" t="str"/>
-      <x:c r="AR37" t="str"/>
-      <x:c r="AS37" s="5" t="str"/>
-      <x:c r="AT37" s="5" t="str"/>
-      <x:c r="AU37" s="5" t="str"/>
-      <x:c r="AV37" t="str"/>
-      <x:c r="AW37" t="str"/>
-      <x:c r="AX37" t="str"/>
+      <x:c r="H37" s="6" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="I37" s="6" t="str"/>
+      <x:c r="J37" s="6" t="str"/>
+      <x:c r="K37" s="6" t="str"/>
+      <x:c r="L37" s="6" t="str"/>
+      <x:c r="M37" s="6" t="str"/>
+      <x:c r="N37" s="6" t="str"/>
+      <x:c r="O37" s="6" t="str"/>
+      <x:c r="P37" s="6" t="str"/>
+      <x:c r="Q37" s="6" t="str"/>
+      <x:c r="R37" s="6" t="str"/>
+      <x:c r="S37" s="6" t="str"/>
+      <x:c r="T37" s="6" t="str"/>
+      <x:c r="U37" s="6" t="str"/>
+      <x:c r="V37" s="6" t="str"/>
+      <x:c r="W37" s="6" t="str"/>
+      <x:c r="X37" s="6" t="str"/>
+      <x:c r="Y37" s="6" t="str"/>
+      <x:c r="Z37" s="6" t="str"/>
+      <x:c r="AA37" s="6" t="str"/>
+      <x:c r="AB37" s="6" t="str"/>
+      <x:c r="AC37" s="6" t="str"/>
+      <x:c r="AD37" s="6" t="str"/>
+      <x:c r="AE37" s="6" t="str"/>
+      <x:c r="AF37" s="6" t="str"/>
+      <x:c r="AG37" s="6" t="str"/>
+      <x:c r="AH37" s="6" t="str"/>
+      <x:c r="AI37" s="6" t="str"/>
+      <x:c r="AJ37" s="6" t="str"/>
+      <x:c r="AK37" s="6" t="str"/>
+      <x:c r="AL37" s="6" t="str"/>
+      <x:c r="AM37" s="6" t="str"/>
+      <x:c r="AN37" s="6" t="str"/>
+      <x:c r="AO37" s="6" t="str"/>
+      <x:c r="AP37" s="6" t="str"/>
+      <x:c r="AQ37" s="6" t="str"/>
+      <x:c r="AR37" s="6" t="str"/>
+      <x:c r="AS37" s="13" t="str"/>
+      <x:c r="AT37" s="13" t="str"/>
+      <x:c r="AU37" s="13" t="str"/>
+      <x:c r="AV37" s="13" t="str"/>
+      <x:c r="AW37" s="13" t="str"/>
+      <x:c r="AX37" s="13" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>6.2</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>README와 실행 방법 최종 정리</x:v>
+        <x:v>사용자 시나리오 테스트</x:v>
       </x:c>
       <x:c r="C38" t="str">
         <x:v>정원식</x:v>
@@ -2941,13 +2941,13 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E38" t="str">
+        <x:v>2026-06-16</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
         <x:v>2026-06-18</x:v>
       </x:c>
-      <x:c r="F38" t="str">
-        <x:v>2026-06-19</x:v>
-      </x:c>
       <x:c r="G38" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H38" t="n">
         <x:v>0</x:v>
@@ -2988,19 +2988,19 @@
       <x:c r="AP38" t="str"/>
       <x:c r="AQ38" t="str"/>
       <x:c r="AR38" t="str"/>
-      <x:c r="AS38" t="str"/>
-      <x:c r="AT38" t="str"/>
+      <x:c r="AS38" s="5" t="str"/>
+      <x:c r="AT38" s="5" t="str"/>
       <x:c r="AU38" s="5" t="str"/>
-      <x:c r="AV38" s="5" t="str"/>
+      <x:c r="AV38" t="str"/>
       <x:c r="AW38" t="str"/>
       <x:c r="AX38" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
-        <x:v>6.3</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>발표 리허설 및 PDF 최종 점검</x:v>
+        <x:v>README와 실행 방법 최종 정리</x:v>
       </x:c>
       <x:c r="C39" t="str">
         <x:v>정원식</x:v>
@@ -3009,13 +3009,13 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="E39" t="str">
+        <x:v>2026-06-18</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
         <x:v>2026-06-19</x:v>
       </x:c>
-      <x:c r="F39" t="str">
-        <x:v>2026-06-21</x:v>
-      </x:c>
       <x:c r="G39" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H39" t="n">
         <x:v>0</x:v>
@@ -3058,78 +3058,146 @@
       <x:c r="AR39" t="str"/>
       <x:c r="AS39" t="str"/>
       <x:c r="AT39" t="str"/>
-      <x:c r="AU39" t="str"/>
+      <x:c r="AU39" s="5" t="str"/>
       <x:c r="AV39" s="5" t="str"/>
-      <x:c r="AW39" s="5" t="str"/>
-      <x:c r="AX39" s="5" t="str"/>
+      <x:c r="AW39" t="str"/>
+      <x:c r="AX39" t="str"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="11" t="str">
+      <x:c r="A40" t="str">
+        <x:v>6.3</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>발표 리허설 및 PDF 최종 점검</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>정원식</x:v>
+      </x:c>
+      <x:c r="D40" s="14" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>2026-06-02</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
+      <x:c r="G40" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H40" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="I40" t="str"/>
+      <x:c r="J40" t="str"/>
+      <x:c r="K40" t="str"/>
+      <x:c r="L40" t="str"/>
+      <x:c r="M40" t="str"/>
+      <x:c r="N40" t="str"/>
+      <x:c r="O40" t="str"/>
+      <x:c r="P40" t="str"/>
+      <x:c r="Q40" t="str"/>
+      <x:c r="R40" t="str"/>
+      <x:c r="S40" t="str"/>
+      <x:c r="T40" t="str"/>
+      <x:c r="U40" t="str"/>
+      <x:c r="V40" t="str"/>
+      <x:c r="W40" t="str"/>
+      <x:c r="X40" t="str"/>
+      <x:c r="Y40" t="str"/>
+      <x:c r="Z40" t="str"/>
+      <x:c r="AA40" t="str"/>
+      <x:c r="AB40" t="str"/>
+      <x:c r="AC40" t="str"/>
+      <x:c r="AD40" t="str"/>
+      <x:c r="AE40" s="15" t="str"/>
+      <x:c r="AF40" s="15" t="str"/>
+      <x:c r="AG40" s="15" t="str"/>
+      <x:c r="AH40" s="15" t="str"/>
+      <x:c r="AI40" s="15" t="str"/>
+      <x:c r="AJ40" s="15" t="str"/>
+      <x:c r="AK40" s="15" t="str"/>
+      <x:c r="AL40" s="15" t="str"/>
+      <x:c r="AM40" s="15" t="str"/>
+      <x:c r="AN40" s="15" t="str"/>
+      <x:c r="AO40" s="15" t="str"/>
+      <x:c r="AP40" s="15" t="str"/>
+      <x:c r="AQ40" s="15" t="str"/>
+      <x:c r="AR40" s="15" t="str"/>
+      <x:c r="AS40" s="15" t="str"/>
+      <x:c r="AT40" s="15" t="str"/>
+      <x:c r="AU40" s="15" t="str"/>
+      <x:c r="AV40" s="15" t="str"/>
+      <x:c r="AW40" s="15" t="str"/>
+      <x:c r="AX40" s="15" t="str"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="11" t="str">
         <x:v>6.4</x:v>
       </x:c>
-      <x:c r="B40" s="11" t="str">
+      <x:c r="B41" s="11" t="str">
         <x:v>최종 발표</x:v>
       </x:c>
-      <x:c r="C40" s="11" t="str">
+      <x:c r="C41" s="11" t="str">
         <x:v>정원식</x:v>
       </x:c>
-      <x:c r="D40" s="11" t="str">
+      <x:c r="D41" s="11" t="str">
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="E40" s="11" t="str">
+      <x:c r="E41" s="11" t="str">
         <x:v>2026-06-22</x:v>
       </x:c>
-      <x:c r="F40" s="11" t="str">
+      <x:c r="F41" s="11" t="str">
         <x:v>2026-06-22</x:v>
       </x:c>
-      <x:c r="G40" s="11" t="n">
+      <x:c r="G41" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H40" s="11" t="n">
+      <x:c r="H41" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I40" s="11" t="str"/>
-      <x:c r="J40" s="11" t="str"/>
-      <x:c r="K40" s="11" t="str"/>
-      <x:c r="L40" s="11" t="str"/>
-      <x:c r="M40" s="11" t="str"/>
-      <x:c r="N40" s="11" t="str"/>
-      <x:c r="O40" s="11" t="str"/>
-      <x:c r="P40" s="11" t="str"/>
-      <x:c r="Q40" s="11" t="str"/>
-      <x:c r="R40" s="11" t="str"/>
-      <x:c r="S40" s="11" t="str"/>
-      <x:c r="T40" s="11" t="str"/>
-      <x:c r="U40" s="11" t="str"/>
-      <x:c r="V40" s="11" t="str"/>
-      <x:c r="W40" s="11" t="str"/>
-      <x:c r="X40" s="11" t="str"/>
-      <x:c r="Y40" s="11" t="str"/>
-      <x:c r="Z40" s="11" t="str"/>
-      <x:c r="AA40" s="11" t="str"/>
-      <x:c r="AB40" s="11" t="str"/>
-      <x:c r="AC40" s="11" t="str"/>
-      <x:c r="AD40" s="11" t="str"/>
-      <x:c r="AE40" s="11" t="str"/>
-      <x:c r="AF40" s="11" t="str"/>
-      <x:c r="AG40" s="11" t="str"/>
-      <x:c r="AH40" s="11" t="str"/>
-      <x:c r="AI40" s="11" t="str"/>
-      <x:c r="AJ40" s="11" t="str"/>
-      <x:c r="AK40" s="11" t="str"/>
-      <x:c r="AL40" s="11" t="str"/>
-      <x:c r="AM40" s="11" t="str"/>
-      <x:c r="AN40" s="11" t="str"/>
-      <x:c r="AO40" s="11" t="str"/>
-      <x:c r="AP40" s="11" t="str"/>
-      <x:c r="AQ40" s="11" t="str"/>
-      <x:c r="AR40" s="11" t="str"/>
-      <x:c r="AS40" s="11" t="str"/>
-      <x:c r="AT40" s="11" t="str"/>
-      <x:c r="AU40" s="11" t="str"/>
-      <x:c r="AV40" s="11" t="str"/>
-      <x:c r="AW40" s="11" t="str"/>
-      <x:c r="AX40" s="11" t="str"/>
+      <x:c r="I41" s="11" t="str"/>
+      <x:c r="J41" s="11" t="str"/>
+      <x:c r="K41" s="11" t="str"/>
+      <x:c r="L41" s="11" t="str"/>
+      <x:c r="M41" s="11" t="str"/>
+      <x:c r="N41" s="11" t="str"/>
+      <x:c r="O41" s="11" t="str"/>
+      <x:c r="P41" s="11" t="str"/>
+      <x:c r="Q41" s="11" t="str"/>
+      <x:c r="R41" s="11" t="str"/>
+      <x:c r="S41" s="11" t="str"/>
+      <x:c r="T41" s="11" t="str"/>
+      <x:c r="U41" s="11" t="str"/>
+      <x:c r="V41" s="11" t="str"/>
+      <x:c r="W41" s="11" t="str"/>
+      <x:c r="X41" s="11" t="str"/>
+      <x:c r="Y41" s="11" t="str"/>
+      <x:c r="Z41" s="11" t="str"/>
+      <x:c r="AA41" s="11" t="str"/>
+      <x:c r="AB41" s="11" t="str"/>
+      <x:c r="AC41" s="11" t="str"/>
+      <x:c r="AD41" s="11" t="str"/>
+      <x:c r="AE41" s="11" t="str"/>
+      <x:c r="AF41" s="11" t="str"/>
+      <x:c r="AG41" s="11" t="str"/>
+      <x:c r="AH41" s="11" t="str"/>
+      <x:c r="AI41" s="11" t="str"/>
+      <x:c r="AJ41" s="11" t="str"/>
+      <x:c r="AK41" s="11" t="str"/>
+      <x:c r="AL41" s="11" t="str"/>
+      <x:c r="AM41" s="11" t="str"/>
+      <x:c r="AN41" s="11" t="str"/>
+      <x:c r="AO41" s="11" t="str"/>
+      <x:c r="AP41" s="11" t="str"/>
+      <x:c r="AQ41" s="11" t="str"/>
+      <x:c r="AR41" s="11" t="str"/>
+      <x:c r="AS41" s="11" t="str"/>
+      <x:c r="AT41" s="11" t="str"/>
+      <x:c r="AU41" s="11" t="str"/>
+      <x:c r="AV41" s="11" t="str"/>
+      <x:c r="AW41" s="11" t="str"/>
+      <x:c r="AX41" s="11" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>